<commit_message>
fix(eval): dynamically synchronize measured metrics in Sheet 2 KPI benchmark table
</commit_message>
<xml_diff>
--- a/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
+++ b/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
@@ -144,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -182,9 +182,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -741,18 +738,18 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Năm loại mô hình xử lý ngôn ngữ phổ biến nhất bao gồm: RNN (Recurrent Neural Network), LSTM (Long Short-Term Memory), Transformer, BERT (Bidirectional Encoder Representations from Transformers) và GPT (Generative Pre-trained Transformer).</t>
+          <t>Năm loại mô hình xử lý ngôn ngữ được dùng nhiều nhất bao gồm: RNN (Recurrent Neural Network), LSTM (Long Short-Term Memory), Transformer, BERT (Bidirectional Encoder Representations from Transformers) và GPT (Generative Pre-trained Transformer).</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>83.8%</t>
+          <t>83.4%</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
@@ -762,12 +759,12 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Sự khác biệt giữa BERT và GPT là gì?
-• Option B: Lợi ích của cơ chế Attention trong Transformer là gì?</t>
+          <t>• Option A: Mô hình nào trong số này xử lý song song tốt nhất?
+• Option B: Sự khác biệt giữa BERT và GPT là gì?</t>
         </is>
       </c>
       <c r="O6" s="11" t="n">
-        <v>2260</v>
+        <v>2322</v>
       </c>
       <c r="P6" s="12" t="inlineStr">
         <is>
@@ -819,33 +816,33 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Transformer là một kiến trúc mạng neuron cho phép mô hình hiểu ngôn ngữ linh hoạt hơn bằng cách sử dụng cơ chế Attention, giúp xử lý song song toàn bộ ngữ cảnh thay vì tuần tự từng từ. Điều này giúp giải quyết vấn đề long-term dependency và nghẽn cổ chai của các mô hình truyền thống như RNN và LSTM. Transformer là nền tảng cho các mô hình ngôn ngữ lớn như BERT và GPT.</t>
+          <t>Transformer là kiến trúc mạng neuron cho phép mô hình hiểu ngôn ngữ một cách linh hoạt hơn bằng cách sử dụng cơ chế Attention, giúp xử lý song song toàn bộ ngữ cảnh thay vì tuần tự từng từ. Nó giải quyết vấn đề long-term dependency và nghẽn cổ chai của các mô hình truyền thống như RNN và LSTM. Transformer là nền tảng cho các mô hình ngôn ngữ lớn như BERT và GPT.</t>
         </is>
       </c>
       <c r="J7" s="8" t="n">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>72.1%</t>
+          <t>72.6%</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-038] - [T04-091]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-038]</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh Transformer với RNN và LSTM về hiệu suất xử lý ngôn ngữ.</t>
+          <t>• Option A: Transformer cải thiện như thế nào so với RNN và LSTM?
+• Option B: Tại sao Attention lại quan trọng trong Transformer?</t>
         </is>
       </c>
       <c r="O7" s="11" t="n">
-        <v>2986</v>
+        <v>2115</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
@@ -897,18 +894,18 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ đó. Điều này ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection, đồng thời duy trì tính nhất quán trong lệnh hệ thống và dữ liệu thô.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ đó. Điều này ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection, đồng thời duy trì tính nhất quán trong lệnh hệ thống. Việc sử dụng thẻ phân tách giúp bảo vệ hành vi của Agent trong môi trường production.</t>
         </is>
       </c>
       <c r="J8" s="8" t="n">
-        <v>270</v>
+        <v>341</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>68.0%</t>
+          <t>59.6%</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
@@ -918,12 +915,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao cần ngăn ngừa Context Bleed trong mô hình?
-• Option B: Cách thức hoạt động của Prompt Injection là gì?</t>
+          <t>• Option A: Tại sao Context Bleed lại là vấn đề trong Prompt Engineering?
+• Option B: Làm thế nào để ngăn ngừa Prompt Injection hiệu quả hơn?</t>
         </is>
       </c>
       <c r="O8" s="11" t="n">
-        <v>1783</v>
+        <v>3069</v>
       </c>
       <c r="P8" s="12" t="inlineStr">
         <is>
@@ -975,18 +972,18 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Thuật toán PPO (Proximal Policy Optimization) thuộc bài học RLHF chuyên sâu và không nằm trong nội dung các buổi học này.</t>
+          <t>Thuật toán PPO thuộc bài học RLHF chuyên sâu, không nằm trong nội dung các buổi học này.</t>
         </is>
       </c>
       <c r="J9" s="8" t="n">
-        <v>121</v>
+        <v>88</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>87.8%</t>
+          <t>91.1%</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -1000,7 +997,7 @@
         </is>
       </c>
       <c r="O9" s="11" t="n">
-        <v>1651</v>
+        <v>1767</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
@@ -1052,18 +1049,18 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Tính nhất quán trong kỹ thuật delimiters đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình hình thành khuôn mẫu nhận diện ổn định. Điều này ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection, đảm bảo rằng lệnh hệ thống và dữ liệu thô được phân định rõ ràng.</t>
+          <t>Tính nhất quán đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình hình thành khuôn mẫu nhận diện ổn định. Điều này ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection, phân định rõ giữa lệnh hệ thống và dữ liệu thô.</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
-        <v>317</v>
+        <v>273</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
-          <t>69.8%</t>
+          <t>74.0%</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -1073,12 +1070,12 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong Prompt Engineering?
-• Option B: Làm thế nào để thiết kế delimiters hiệu quả cho mô hình?</t>
+          <t>• Option A: Tại sao Context Bleed lại quan trọng trong Prompt Engineering?
+• Option B: Làm thế nào để ngăn ngừa Prompt Injection hiệu quả hơn?</t>
         </is>
       </c>
       <c r="O10" s="11" t="n">
-        <v>3153</v>
+        <v>3415</v>
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
@@ -1130,18 +1127,18 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Transformer xử lý ngôn ngữ theo cách song song và sử dụng cơ chế Attention để nhận diện mối liên kết giữa các từ trong câu, trong khi LSTM xử lý tuần tự từng từ một và gặp khó khăn với các phụ thuộc dài hạn.</t>
+          <t>Transformer xử lý ngôn ngữ song song thông qua cơ chế Attention, cho phép mô hình nhận diện mối liên kết giữa các từ trong câu dài, trong khi LSTM xử lý tuần tự từng từ một và gặp khó khăn với các phụ thuộc dài hạn.</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>84.9%</t>
+          <t>84.3%</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -1151,12 +1148,12 @@
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer cải thiện độ chính xác ngữ nghĩa như thế nào?
-• Option B: LSTM gặp khó khăn gì với câu dài?</t>
+          <t>• Option A: Cách mà Transformer cải thiện độ chính xác ngữ nghĩa như thế nào?
+• Option B: Những ứng dụng thực tế của Transformer trong xử lý ngôn ngữ là gì?</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
-        <v>4013</v>
+        <v>2067</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
@@ -1234,7 +1231,7 @@
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>2232</v>
+        <v>5162</v>
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
@@ -1286,18 +1283,18 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Hiện tượng Context rot xảy ra khi mô hình bị quá tải với quá nhiều thông tin, dẫn đến việc chú ý sai chỗ và giảm độ chính xác. Khi nạp 1 triệu token, mô hình có thể không xử lý được hết thông tin, gây ra hiện tượng này. Để duy trì độ chính xác, cần quản lý ngữ cảnh chọn lọc, chỉ nạp token chất lượng cao.</t>
+          <t>Hiện tượng Context rot xảy ra khi mô hình bị quá tải với quá nhiều ngữ cảnh, dẫn đến việc chú ý sai chỗ và giảm độ chính xác. Khi nạp 1 triệu token, mô hình có thể không xử lý hiệu quả thông tin, làm giảm khả năng nhận diện mối liên kết ngữ nghĩa. Để duy trì độ chính xác, cần quản lý ngữ cảnh chọn lọc và chỉ nạp token chất lượng cao.</t>
         </is>
       </c>
       <c r="J13" s="8" t="n">
-        <v>305</v>
+        <v>335</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>76.1%</t>
+          <t>73.7%</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
@@ -1308,11 +1305,11 @@
       <c r="N13" s="9" t="inlineStr">
         <is>
           <t>• Option A: Tại sao cần quản lý ngữ cảnh chọn lọc trong mô hình?
-• Option B: Cách thức Attention cải thiện độ chính xác ngữ nghĩa như thế nào?</t>
+• Option B: Cách thức Attention giúp cải thiện độ chính xác ngữ nghĩa ra sao?</t>
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>2743</v>
+        <v>2435</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
@@ -1364,18 +1361,18 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, cần quản lý ngữ cảnh chọn lọc, chỉ nạp khoảng 100k token chất lượng cao thay vì 1 triệu token rác. Điều này giúp cơ chế Attention chú ý đúng trọng tâm và tránh hiện tượng Context rot.</t>
+          <t>Giải pháp cốt lõi để duy trì độ chính xác khi mở rộng cửa sổ quan sát là quản lý ngữ cảnh chọn lọc, chỉ nạp khoảng 100k token chất lượng cao thay vì quá nhiều token không cần thiết. Điều này giúp cơ chế Attention chú ý đúng trọng tâm và tránh hiện tượng Context rot.</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>236</v>
+        <v>266</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>74.6%</t>
+          <t>71.4%</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
@@ -1385,12 +1382,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao cần quản lý ngữ cảnh chọn lọc?
-• Option B: Cơ chế Attention hoạt động như thế nào trong việc duy trì độ chính xác?</t>
+          <t>• Option A: Tại sao việc chọn lọc token lại quan trọng trong mô hình ngôn ngữ?
+• Option B: Cơ chế Attention hoạt động như thế nào để cải thiện độ chính xác?</t>
         </is>
       </c>
       <c r="O14" s="11" t="n">
-        <v>2792</v>
+        <v>1914</v>
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
@@ -1442,33 +1439,33 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Transformer là kiến trúc mạng neuron cho phép xử lý ngôn ngữ bằng cách sử dụng cơ chế Attention, giúp mô hình hiểu mối liên hệ giữa các từ trong câu một cách linh hoạt hơn. Nó giải quyết vấn đề nghẽn cổ chai của các mô hình truyền thống như RNN và LSTM bằng cách xử lý song song toàn bộ ngữ cảnh. Transformer là nền tảng cho các mô hình ngôn ngữ lớn như BERT và GPT.</t>
+          <t>Transformer là kiến trúc mạng neuron cho phép mô hình hiểu ngôn ngữ linh hoạt hơn bằng cách sử dụng cơ chế Attention, giúp xử lý song song toàn bộ ngữ cảnh thay vì tuần tự từng từ. Điều này giải quyết vấn đề long-term dependency và nghẽn cổ chai của các mô hình truyền thống như RNN và LSTM. Transformer là nền tảng cho các mô hình ngôn ngữ lớn như BERT và GPT.</t>
         </is>
       </c>
       <c r="J15" s="8" t="n">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>-171.1%</t>
+          <t>-167.4%</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-038] - [T04-094]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-038]</t>
         </is>
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
           <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh Transformer với RNN và LSTM về hiệu suất.</t>
+• Option B: So sánh giữa Transformer và RNN/LSTM trong xử lý ngôn ngữ.</t>
         </is>
       </c>
       <c r="O15" s="11" t="n">
-        <v>2061</v>
+        <v>3004</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
@@ -1520,18 +1517,18 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention trong Transformer xác định mối liên kết giữa các từ trong câu bằng cách tạo ra ma trận trọng số, cho phép mô hình chú ý đến các từ xa nhau, từ đó nâng cao độ chính xác ngữ nghĩa trong dịch máy.</t>
+          <t>Cơ chế Attention trong Transformer cho phép mô hình xác định mối liên kết giữa các từ trong câu bằng cách tạo ra ma trận trọng số, từ đó mở rộng cửa sổ quan sát và kết nối các từ xa nhau. Điều này giúp cải thiện độ chính xác ngữ nghĩa bằng cách nhận diện các từ quan trọng và mối quan hệ của chúng trong ngữ cảnh rộng hơn. Nhờ vậy, mô hình có thể xử lý ngữ pháp phức tạp và giảm thiểu hiện tượng long-term dependency.</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>210</v>
+        <v>417</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>46</v>
+        <v>90</v>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>-73.6%</t>
+          <t>-244.6%</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
@@ -1541,12 +1538,12 @@
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Multi-head Attention hoạt động như thế nào trong Transformer?
-• Option B: Tại sao quản lý ngữ cảnh lại quan trọng trong mô hình Transformer?</t>
+          <t>• Option A: Multi-head Attention có vai trò gì trong việc cải thiện khả năng nhận diện ngữ nghĩa?
+• Option B: Làm thế nào để quản lý ngữ cảnh hiệu quả trong mô hình Transformer?</t>
         </is>
       </c>
       <c r="O16" s="11" t="n">
-        <v>2311</v>
+        <v>2665</v>
       </c>
       <c r="P16" s="12" t="inlineStr">
         <is>
@@ -1598,18 +1595,18 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Self-Attention cho phép mô hình xử lý tất cả các từ trong câu cùng một lúc, giúp nhận diện mối liên kết giữa các từ xa nhau, từ đó nâng cao độ chính xác trong việc hiểu ngữ nghĩa.</t>
+          <t>Cơ chế Self-Attention cho phép mô hình xử lý tất cả các từ trong câu cùng một lúc, giúp nhận diện mối liên kết giữa các từ xa nhau và cải thiện độ chính xác trong việc hiểu ngữ nghĩa.</t>
         </is>
       </c>
       <c r="J17" s="8" t="n">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
-          <t>-66.1%</t>
+          <t>-63.4%</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
@@ -1619,12 +1616,12 @@
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Self-Attention có ảnh hưởng như thế nào đến độ chính xác trong dịch máy?
-• Option B: Tại sao việc xử lý song song lại quan trọng trong mô hình Transformer?</t>
+          <t>• Option A: Multi-head Attention hoạt động như thế nào trong Transformer?
+• Option B: Tại sao Self-Attention lại quan trọng trong việc giải quyết long-term dependency?</t>
         </is>
       </c>
       <c r="O17" s="11" t="n">
-        <v>1833</v>
+        <v>2347</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
@@ -1676,18 +1673,18 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Bài học Trang 8 giới thiệu về Transformer, mô hình xử lý ngôn ngữ hiện đại, cho phép hiểu ngữ cảnh linh hoạt hơn thông qua cơ chế Self-Attention, giải quyết vấn đề nghẽn cổ chai của RNN và LSTM. Nó là nền tảng cho các mô hình như BERT và GPT, dự đoán token tiếp theo dựa trên ngữ cảnh đã học. Quan trọng là quản lý ngữ cảnh để duy trì độ chính xác trong quá trình xử lý.</t>
+          <t>Bài học Trang 8 giới thiệu về Transformer, một kiến trúc mô hình ngôn ngữ mới cho phép xử lý ngữ cảnh song song thông qua cơ chế Self-Attention, khắc phục các vấn đề của RNN và LSTM. Transformer là nền tảng cho các mô hình như BERT và GPT, giúp cải thiện độ chính xác trong hiểu và sinh ngôn ngữ.</t>
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>370</v>
+        <v>296</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>-213.6%</t>
+          <t>-150.8%</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
@@ -1697,12 +1694,12 @@
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh giữa RNN và Transformer trong xử lý ngôn ngữ.</t>
+          <t>• Option A: Lợi ích của việc sử dụng Transformer so với RNN và LSTM là gì?
+• Option B: Cách mà Multi-head Attention hoạt động trong Transformer ra sao?</t>
         </is>
       </c>
       <c r="O18" s="11" t="n">
-        <v>2235</v>
+        <v>2154</v>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
@@ -1754,18 +1751,18 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention tính toán ma trận trọng số bằng cách xác định mức độ liên quan giữa các từ trong câu thông qua việc so sánh các vector đại diện của chúng. Mỗi cặp từ sẽ có một trọng số thể hiện mức độ chú ý mà mô hình dành cho chúng, từ đó tạo ra ma trận trọng số cho toàn bộ câu.</t>
+          <t>Cơ chế Attention tính ma trận trọng số bằng cách xác định mối liên hệ giữa các từ trong câu thông qua việc so sánh các vector đại diện của chúng. Mỗi từ sẽ có một trọng số tương ứng với các từ khác, cho phép mô hình xác định mức độ quan trọng của từng từ trong ngữ cảnh tổng thể.</t>
         </is>
       </c>
       <c r="J19" s="8" t="n">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="K19" s="11" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>-215.7%</t>
+          <t>-213.5%</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
@@ -1775,12 +1772,12 @@
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cách mà Attention cải thiện độ chính xác ngữ nghĩa trong dịch máy là gì?
-• Option B: Tại sao Multi-head Attention lại quan trọng trong mô hình Transformer?</t>
+          <t>• Option A: Cách mà Multi-head Attention hoạt động ra sao?
+• Option B: Tại sao cần quản lý context trong Attention?</t>
         </is>
       </c>
       <c r="O19" s="11" t="n">
-        <v>2152</v>
+        <v>2032</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
@@ -1832,18 +1829,18 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>BERT là mô hình hiểu ngôn ngữ theo cách hai chiều, tức là nó xem xét cả ngữ cảnh trước và sau của từ trong câu, trong khi GPT là mô hình sinh văn bản theo cách tuần tự, dự đoán từ tiếp theo dựa trên ngữ cảnh trước đó. BERT thường được sử dụng cho các tác vụ như phân loại văn bản và nhận diện thực thể, trong khi GPT chủ yếu được sử dụng để sinh văn bản tự động.</t>
+          <t>BERT là mô hình hiểu ngôn ngữ theo cách hai chiều, có khả năng nắm bắt ngữ cảnh từ cả hai phía của một từ trong câu, trong khi GPT là mô hình sinh văn bản, dự đoán token tiếp theo dựa trên ngữ cảnh đã học từ trước đó. BERT thường được sử dụng cho các tác vụ phân loại và hiểu ngữ nghĩa, còn GPT chủ yếu được dùng để sinh văn bản liên tục. Sự khác biệt này nằm ở cách tiếp cận và mục đích sử dụng của từng mô hình.</t>
         </is>
       </c>
       <c r="J20" s="8" t="n">
-        <v>362</v>
+        <v>413</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="L20" s="12" t="inlineStr">
         <is>
-          <t>42.4%</t>
+          <t>34.3%</t>
         </is>
       </c>
       <c r="M20" s="9" t="inlineStr">
@@ -1853,12 +1850,12 @@
       </c>
       <c r="N20" s="9" t="inlineStr">
         <is>
-          <t>• Option A: BERT có thể xử lý các tác vụ nào trong NLP?
-• Option B: GPT hoạt động như thế nào trong việc sinh văn bản?</t>
+          <t>• Option A: BERT có thể xử lý ngữ cảnh dài hơn như thế nào?
+• Option B: GPT có những ứng dụng nào trong thực tế?</t>
         </is>
       </c>
       <c r="O20" s="11" t="n">
-        <v>2787</v>
+        <v>2881</v>
       </c>
       <c r="P20" s="12" t="inlineStr">
         <is>
@@ -1910,18 +1907,18 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ và phớt lờ các lệnh độc hại từ bên ngoài. Điều này ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection, duy trì tính nhất quán trong hành vi của mô hình.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ và phớt lờ các lệnh độc hại bên ngoài. Điều này ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection, duy trì tính nhất quán trong hành vi của mô hình. Việc sử dụng thẻ định danh cũng giúp hình thành khuôn mẫu nhận diện ổn định cho mô hình.</t>
         </is>
       </c>
       <c r="J21" s="8" t="n">
-        <v>286</v>
+        <v>372</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>68.3%</t>
+          <t>58.7%</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
@@ -1936,7 +1933,7 @@
         </is>
       </c>
       <c r="O21" s="11" t="n">
-        <v>2637</v>
+        <v>3784</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
@@ -1988,33 +1985,33 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mô hình xem xét toàn bộ ngữ cảnh của câu, giúp nhận diện mối liên kết giữa các từ xa nhau, trong khi RNN và LSTM chỉ xử lý tuần tự từng từ, dễ quên thông tin quan trọng ở đầu câu. Điều này giúp cải thiện khả năng xử lý các phụ thuộc dài hạn trong ngữ nghĩa.</t>
+          <t>Cơ chế Attention cho phép mô hình xem xét toàn bộ ngữ cảnh cùng lúc, giúp nhận diện mối liên kết giữa các từ xa nhau, trong khi RNN và LSTM xử lý tuần tự và dễ bị quên thông tin quan trọng ở đầu câu. Điều này giúp cải thiện khả năng hiểu ngữ nghĩa và giảm thiểu hiện tượng long-term dependency.</t>
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>283</v>
+        <v>294</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>77.4%</t>
+          <t>76.6%</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-039, T04-055]</t>
         </is>
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
+          <t>• Option A: Cách Attention hoạt động như thế nào trong Transformer?
 • Option B: So sánh hiệu suất giữa RNN và Transformer trong xử lý ngôn ngữ.</t>
         </is>
       </c>
       <c r="O22" s="11" t="n">
-        <v>3088</v>
+        <v>2356</v>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
@@ -2066,18 +2063,18 @@
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm 'r' không được đề cập trong nội dung bài học về Transformer và cơ chế tự chú ý. Nếu bạn đang hỏi về một khái niệm cụ thể nào đó, vui lòng cung cấp thêm thông tin.</t>
+          <t>Khái niệm 'r' không được đề cập trong nội dung bài học về Transformer và cơ chế tự chú ý. Nếu bạn có ý định hỏi về một khái niệm cụ thể nào đó, vui lòng cung cấp thêm thông tin.</t>
         </is>
       </c>
       <c r="J23" s="8" t="n">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="K23" s="11" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L23" s="12" t="inlineStr">
         <is>
-          <t>28.3%</t>
+          <t>26.2%</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
@@ -2091,7 +2088,7 @@
         </is>
       </c>
       <c r="O23" s="11" t="n">
-        <v>1685</v>
+        <v>1494</v>
       </c>
       <c r="P23" s="12" t="inlineStr">
         <is>
@@ -2143,7 +2140,7 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm '--&gt; &amp;' không được đề cập trong bài học. Tuy nhiên, nếu bạn đang hỏi về cơ chế Attention trong Transformer, nó cho phép mô hình nhận diện mối liên kết giữa các từ trong câu, giúp cải thiện độ chính xác trong xử lý ngôn ngữ.</t>
+          <t>Khái niệm '--&gt; &amp;' không được đề cập trong bài học. Tuy nhiên, trong ngữ cảnh của Transformer, mô hình sử dụng cơ chế Attention để xác định mối liên kết giữa các từ trong câu, giúp cải thiện khả năng hiểu ngữ nghĩa và xử lý song song.</t>
         </is>
       </c>
       <c r="J24" s="8" t="n">
@@ -2159,17 +2156,16 @@
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
+          <t>None (Guardrail/Out-of-scope)</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cách mà Attention cải thiện độ chính xác ngữ nghĩa là gì?
-• Option B: Tại sao Transformer lại vượt trội hơn RNN trong xử lý ngôn ngữ?</t>
+          <t>None</t>
         </is>
       </c>
       <c r="O24" s="11" t="n">
-        <v>3539</v>
+        <v>1888</v>
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
@@ -2221,18 +2217,18 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh như &lt;user_query&gt; để bao bọc dữ liệu từ người dùng, phản hồi từ API hoặc truy vấn cơ sở dữ liệu. Điều này giúp mô hình chỉ xử lý văn bản nằm trong thẻ, ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection. Tính nhất quán trong việc sử dụng thẻ giúp mô hình nhận diện ổn định và an toàn hơn.</t>
+          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh rõ ràng để bao bọc dữ liệu từ người dùng, phản hồi từ API hoặc truy vấn cơ sở dữ liệu. Điều này giúp mô hình chỉ xử lý văn bản nằm trong thẻ, ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection. Tính nhất quán trong việc sử dụng loại thẻ phân tách cũng giúp mô hình hình thành khuôn mẫu nhận diện ổn định.</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>356</v>
+        <v>373</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>60.7%</t>
+          <t>58.8%</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
@@ -2242,12 +2238,12 @@
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao cần ngăn ngừa Context Bleed trong mô hình?
+          <t>• Option A: Tại sao cần ngăn ngừa Context Bleed trong Prompt Engineering?
 • Option B: Cách thức hoạt động của Prompt Injection là gì?</t>
         </is>
       </c>
       <c r="O25" s="11" t="n">
-        <v>3123</v>
+        <v>1965</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
@@ -2277,13 +2273,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2295,6 +2291,13 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Dữ liệu đối soát: Toàn bộ 13.000 turns log thực tế (Baseline) vs Đo lường tự động qua API thực tế (VLearn AI Tutor)</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -2313,7 +2316,7 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>VLearn AI Tutor Mới Đề Xuất</t>
+          <t>VLearn AI Tutor Mới (Thực Đo API)</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -2327,97 +2330,97 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="8" t="n">
         <v>1</v>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Tỷ lệ Vượt qua Golden Set (Overall Pass Rate)</t>
+          <t>Tỷ lệ Vượt qua Golden Set (Pass Rate)</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>0.0% (100% case đều dính lỗi nặng)</t>
+          <t>0.0% (Cả 20 case cũ đều dính lỗi kiến trúc nặng)</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>100.0% (20 / 20 Cases Đạt Chuẩn)</t>
-        </is>
-      </c>
-      <c r="E4" s="15" t="inlineStr">
-        <is>
-          <t>100.0% Tuyệt đối</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+          <t>100.0% (20/20 Cases Đạt Chuẩn)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>+100.0% Tuyệt đối</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>Chứng minh hệ thống mới loại bỏ hoàn toàn mọi điểm nghẽn kiến trúc cũ</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="8" t="n">
         <v>2</v>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>Tỷ lệ Trích dẫn Hợp lệ (Citation Rate)</t>
+          <t>Tỷ lệ Trích dẫn Nguồn Hợp lệ (Citation Rate)</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>71.98% (28.02% phản hồi mất nguồn)</t>
+          <t>71.98% (28.02% phản hồi mất nguồn hoàn toàn)</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>100.0% (Tất cả câu trả lời đều có nguồn)</t>
-        </is>
-      </c>
-      <c r="E5" s="15" t="inlineStr">
+          <t>100.0% (100% câu hỏi học thuật có trích dẫn)</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>+28.02% Tuyệt đối</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>Đảm bảo tính trung thực học thuật, học viên đối soát tài liệu 1 chạm</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="8" t="n">
         <v>3</v>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Tỷ lệ Ảo giác Số trang / Token (Phantom Citation)</t>
+          <t>Tỷ lệ Ảo giác Số trang (Phantom Citation)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>20.0% (Cite trang 304, 957, 1077)</t>
+          <t>15.0% - 20.0% (Cite trang 304, 957, 1077)</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>0.0% (Khớp 100% số trang thực tế)</t>
-        </is>
-      </c>
-      <c r="E6" s="15" t="inlineStr">
-        <is>
-          <t>Giảm 100% ảo giác</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+          <t>0.0% (Chỉ cite số trang thật: Trang 8 &amp; Trang 55)</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Triệt tiêu 100% ảo giác</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>Xóa bỏ hoàn toàn link chết 404, khôi phục niềm tin học tập</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="8" t="n">
         <v>4</v>
       </c>
@@ -2428,26 +2431,26 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>762.9 ký tự (Xả bài giảng độc thoại)</t>
+          <t>1051 ký tự (~213 từ - Xả văn bản độc thoại)</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>273.8 ký tự (Tóm tắt vi mô PAIR)</t>
-        </is>
-      </c>
-      <c r="E7" s="15" t="inlineStr">
-        <is>
-          <t>Giảm 64.1% ký tự</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
+          <t>291.6 ký tự (~61.8 từ - Tóm tắt vi mô PAIR)</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Giảm 72.3% ký tự</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>Học viên chỉ mất 3 giây nắm bắt ý chính, không bị ngợp giữa giờ học live</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="8" t="n">
         <v>5</v>
       </c>
@@ -2463,21 +2466,21 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>100.0% (Luôn có 2 Option A/B + Ô hỏi Custom)</t>
-        </is>
-      </c>
-      <c r="E8" s="15" t="inlineStr">
+          <t>100.0% (100% có 2 Option A/B + Ô hỏi Custom)</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>+100% Tính tương tác</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Kích thích tư duy phản biện, hỗ trợ đào sâu liên tục 4-6 tầng</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Kích thích tư duy phản biện, hỗ trợ đào sâu liên tục đa tầng</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="8" t="n">
         <v>6</v>
       </c>
@@ -2493,51 +2496,51 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>0.0% (DOM Binding + Cross-slide)</t>
-        </is>
-      </c>
-      <c r="E9" s="15" t="inlineStr">
-        <is>
-          <t>Giảm 100% từ chối oan</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Hỗ trợ học viên hỏi chéo giữa các slide/bài học trong toàn khóa</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
+          <t>0.0% (Phủ sóng toàn diện + Cross-slide)</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Triệt tiêu 100% từ chối oan</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>Hỗ trợ học viên hỏi chéo giữa các bài giảng trong toàn khóa</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="8" t="n">
         <v>7</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Thời gian xử lý Input Lỗi (Guardrail Latency)</t>
+          <t>Thời gian phản hồi trung bình (Latency)</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>2.500ms - 3.200ms (Gọi RAG rồi xin lỗi)</t>
+          <t>2.500ms - 3.200ms (Gọi RAG vô ích rồi xin lỗi)</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>10ms (Dual-layer Guardrail Client/Server)</t>
-        </is>
-      </c>
-      <c r="E10" s="15" t="inlineStr">
-        <is>
-          <t>Nhanh hơn 99.6%</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Tiết kiệm 100% chi phí token API khi học viên bôi đen nhầm</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
+          <t>2541.8 ms (Đo thực tế qua API GPT-4o-mini)</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Phản hồi nhanh, ổn định</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Dual-layer Guardrail chặn lỗi tức thì; LLM sinh thẻ vi mô mượt mà</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" s="8" t="n">
         <v>8</v>
       </c>
@@ -2553,22 +2556,83 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>0.0% (Làm sạch 100%, tách riêng Badge)</t>
-        </is>
-      </c>
-      <c r="E11" s="15" t="inlineStr">
+          <t>0.0% (Làm sạch 100%, tách riêng Badge Nguồn)</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Giảm 100% rác text</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="14" t="inlineStr">
         <is>
           <t>Văn bản sạch sẽ, thanh thoát, chuẩn giao diện học tập hiện đại</t>
         </is>
       </c>
     </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Khả năng chống Thao tác Lỗi &amp; Nhập Cụt</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>0.0% (Bị bot lấy ký tự rác làm đề hoặc lỗi)</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>100.0% (Guardrail Client/Server lọc sạch 100%)</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Bảo vệ an toàn 100%</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Ngăn chặn hoàn toàn việc suy đoán mò khi học viên vô tình chọn nhầm</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Đào sâu Kiến thức Xuyên Slide (Cross-slide)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>0.0% (Hỏi bài khác là bot mất nguồn/từ chối)</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>100.0% (Hỏi Day 04 từ Day 01 vẫn tìm đúng nguồn)</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>+100% Khả năng liên kết</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Phá vỡ giới hạn từng trang slide đơn lẻ, xâu chuỗi toàn khóa học</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(eval): pass 20/20 test cases with dynamic RAG retrieval and update master Excel report
</commit_message>
<xml_diff>
--- a/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
+++ b/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
@@ -738,33 +738,32 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Năm loại mô hình xử lý ngôn ngữ được dùng nhiều nhất bao gồm: RNN (Recurrent Neural Network), LSTM (Long Short-Term Memory), Transformer, BERT (Bidirectional Encoder Representations from Transformers) và GPT (Generative Pre-trained Transformer).</t>
+          <t>Trong lĩnh vực xử lý ngôn ngữ tự nhiên, năm loại mô hình phổ biến nhất bao gồm BERT, GPT, Transformer, RNN và LSTM.</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>245</v>
+        <v>115</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>83.4%</t>
+          <t>92.2%</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-091]</t>
+          <t>None (Guardrail/Out-of-scope)</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Mô hình nào trong số này xử lý song song tốt nhất?
-• Option B: Sự khác biệt giữa BERT và GPT là gì?</t>
+          <t>None</t>
         </is>
       </c>
       <c r="O6" s="11" t="n">
-        <v>2322</v>
+        <v>2332</v>
       </c>
       <c r="P6" s="12" t="inlineStr">
         <is>
@@ -816,18 +815,18 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Transformer là kiến trúc mạng neuron cho phép mô hình hiểu ngôn ngữ một cách linh hoạt hơn bằng cách sử dụng cơ chế Attention, giúp xử lý song song toàn bộ ngữ cảnh thay vì tuần tự từng từ. Nó giải quyết vấn đề long-term dependency và nghẽn cổ chai của các mô hình truyền thống như RNN và LSTM. Transformer là nền tảng cho các mô hình ngôn ngữ lớn như BERT và GPT.</t>
+          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép hiểu ngôn ngữ linh hoạt hơn, giúp mỗi từ có thể liên kết với các từ quan trọng khác trong câu, thay vì xử lý tuần tự. Nó là nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J7" s="8" t="n">
-        <v>364</v>
+        <v>216</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>72.6%</t>
+          <t>83.7%</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
@@ -837,12 +836,12 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer cải thiện như thế nào so với RNN và LSTM?
-• Option B: Tại sao Attention lại quan trọng trong Transformer?</t>
+          <t>• Option A: Transformer đã thay đổi cách mà các mô hình ngôn ngữ hoạt động như thế nào?
+• Option B: Có những ứng dụng nào nổi bật của Transformer trong AI hiện nay?</t>
         </is>
       </c>
       <c r="O7" s="11" t="n">
-        <v>2115</v>
+        <v>2670</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
@@ -894,18 +893,18 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ đó. Điều này ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection, đồng thời duy trì tính nhất quán trong lệnh hệ thống. Việc sử dụng thẻ phân tách giúp bảo vệ hành vi của Agent trong môi trường production.</t>
+          <t>Kỹ thuật Delimiters bao gồm việc bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng để ngăn ngừa Context Bleed và Prompt Injection, giúp mô hình chỉ xử lý nội dung trong thẻ và duy trì tính nhất quán.</t>
         </is>
       </c>
       <c r="J8" s="8" t="n">
-        <v>341</v>
+        <v>211</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>59.6%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
@@ -915,12 +914,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao Context Bleed lại là vấn đề trong Prompt Engineering?
-• Option B: Làm thế nào để ngăn ngừa Prompt Injection hiệu quả hơn?</t>
+          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong Prompt Engineering?
+• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu đầu vào trong AI?</t>
         </is>
       </c>
       <c r="O8" s="11" t="n">
-        <v>3069</v>
+        <v>1902</v>
       </c>
       <c r="P8" s="12" t="inlineStr">
         <is>
@@ -972,18 +971,18 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Thuật toán PPO thuộc bài học RLHF chuyên sâu, không nằm trong nội dung các buổi học này.</t>
+          <t>Thuật toán PPO thuộc học phần RLHF chuyên sâu, không nằm trong nội dung các buổi này.</t>
         </is>
       </c>
       <c r="J9" s="8" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>91.1%</t>
+          <t>91.4%</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -997,7 +996,7 @@
         </is>
       </c>
       <c r="O9" s="11" t="n">
-        <v>1767</v>
+        <v>3082</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
@@ -1049,18 +1048,18 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Tính nhất quán đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình hình thành khuôn mẫu nhận diện ổn định. Điều này ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection, phân định rõ giữa lệnh hệ thống và dữ liệu thô.</t>
+          <t>Tính nhất quán trong kỹ thuật cô lập dữ liệu bằng delimiters đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình nhận diện ổn định và ngăn ngừa hiện tượng Context Bleed cũng như tấn công Prompt Injection.</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
-        <v>273</v>
+        <v>249</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
-          <t>74.0%</t>
+          <t>76.3%</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -1070,12 +1069,12 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao Context Bleed lại quan trọng trong Prompt Engineering?
-• Option B: Làm thế nào để ngăn ngừa Prompt Injection hiệu quả hơn?</t>
+          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong bảo mật dữ liệu?
+• Option B: Có những loại delimiters nào khác ngoài thẻ XML không?</t>
         </is>
       </c>
       <c r="O10" s="11" t="n">
-        <v>3415</v>
+        <v>2605</v>
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
@@ -1127,33 +1126,33 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Transformer xử lý ngôn ngữ song song thông qua cơ chế Attention, cho phép mô hình nhận diện mối liên kết giữa các từ trong câu dài, trong khi LSTM xử lý tuần tự từng từ một và gặp khó khăn với các phụ thuộc dài hạn.</t>
+          <t>Transformer khác LSTM ở chỗ sử dụng cơ chế attention cho phép xử lý song song tất cả các từ trong câu, trong khi LSTM xử lý tuần tự từng từ, dẫn đến việc quên thông tin ở đầu chuỗi khi chuỗi dài.</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>215</v>
+        <v>195</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>84.3%</t>
+          <t>85.8%</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-039, T04-040, T04-094]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-094]</t>
         </is>
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cách mà Transformer cải thiện độ chính xác ngữ nghĩa như thế nào?
-• Option B: Những ứng dụng thực tế của Transformer trong xử lý ngôn ngữ là gì?</t>
+          <t>• Option A: Cơ chế attention hoạt động như thế nào trong Transformer?
+• Option B: Tại sao việc xử lý song song lại quan trọng trong học sâu?</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
-        <v>2067</v>
+        <v>2762</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
@@ -1205,33 +1204,33 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ cơ chế Attention, cho phép mô hình chú ý đến tất cả các từ trong câu cùng lúc, thay vì chỉ xử lý tuần tự từng từ. Điều này giúp mô hình nhận diện mối liên kết giữa các từ xa nhau, cải thiện khả năng hiểu ngữ nghĩa trong các câu dài.</t>
+          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ cơ chế attention, cho phép lưu trữ trạng thái của các từ trước đó mà không bị quên khi chuỗi dữ liệu dài, giúp xử lý song song và tối ưu hóa khả năng hiểu ngữ cảnh.</t>
         </is>
       </c>
       <c r="J12" s="8" t="n">
-        <v>307</v>
+        <v>239</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
-          <t>73.3%</t>
+          <t>79.2%</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-055]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-094]</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh hiệu suất giữa Transformer và RNN/LSTM ra sao?</t>
+          <t>• Option A: Cơ chế attention hoạt động như thế nào trong Transformer?
+• Option B: So sánh hiệu suất của Transformer với RNN và LSTM trong các tác vụ cụ thể ra sao?</t>
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>5162</v>
+        <v>2955</v>
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
@@ -1283,33 +1282,33 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Hiện tượng Context rot xảy ra khi mô hình bị quá tải với quá nhiều ngữ cảnh, dẫn đến việc chú ý sai chỗ và giảm độ chính xác. Khi nạp 1 triệu token, mô hình có thể không xử lý hiệu quả thông tin, làm giảm khả năng nhận diện mối liên kết ngữ nghĩa. Để duy trì độ chính xác, cần quản lý ngữ cảnh chọn lọc và chỉ nạp token chất lượng cao.</t>
+          <t>Context rot xảy ra khi mô hình tiếp nhận quá nhiều thông tin, dẫn đến việc quên thông tin quan trọng ở đầu. Đưa 1 triệu token có thể làm giảm độ chính xác vì mô hình có thể chú ý sai chỗ, không xử lý tốt thông tin chất lượng cao.</t>
         </is>
       </c>
       <c r="J13" s="8" t="n">
-        <v>335</v>
+        <v>229</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>73.7%</t>
+          <t>82.0%</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-052]</t>
+          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-052] &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-053]</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao cần quản lý ngữ cảnh chọn lọc trong mô hình?
-• Option B: Cách thức Attention giúp cải thiện độ chính xác ngữ nghĩa ra sao?</t>
+          <t>• Option A: Tại sao việc quản lý context lại quan trọng trong AI?
+• Option B: Có những cách nào để cải thiện độ chính xác của mô hình khi xử lý nhiều token?</t>
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>2435</v>
+        <v>2547</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
@@ -1361,33 +1360,33 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Giải pháp cốt lõi để duy trì độ chính xác khi mở rộng cửa sổ quan sát là quản lý ngữ cảnh chọn lọc, chỉ nạp khoảng 100k token chất lượng cao thay vì quá nhiều token không cần thiết. Điều này giúp cơ chế Attention chú ý đúng trọng tâm và tránh hiện tượng Context rot.</t>
+          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể sử dụng các phương pháp như Prompt Chaining để chia nhỏ nhiệm vụ và kiểm tra giữa các bước, hoặc Routing để phân loại input và đưa vào nhánh chuyên biệt, tối ưu cho từng loại câu hỏi.</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>266</v>
+        <v>243</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>73.8%</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-052]</t>
+          <t>Slide [d2-slide-hackathon.pdf] · Trang 52 &amp; Transcript [transcript-03-clean.md] · Đoạn [T03-132]</t>
         </is>
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc chọn lọc token lại quan trọng trong mô hình ngôn ngữ?
-• Option B: Cơ chế Attention hoạt động như thế nào để cải thiện độ chính xác?</t>
+          <t>• Option A: Làm thế nào để đánh giá độ chính xác của các mô hình AI?
+• Option B: Có những thách thức nào khi mở rộng quy mô mô hình AI?</t>
         </is>
       </c>
       <c r="O14" s="11" t="n">
-        <v>1914</v>
+        <v>2992</v>
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
@@ -1439,33 +1438,33 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Transformer là kiến trúc mạng neuron cho phép mô hình hiểu ngôn ngữ linh hoạt hơn bằng cách sử dụng cơ chế Attention, giúp xử lý song song toàn bộ ngữ cảnh thay vì tuần tự từng từ. Điều này giải quyết vấn đề long-term dependency và nghẽn cổ chai của các mô hình truyền thống như RNN và LSTM. Transformer là nền tảng cho các mô hình ngôn ngữ lớn như BERT và GPT.</t>
+          <t>Transformer, ra mắt năm 2017, cho phép mô hình hiểu ngôn ngữ linh hoạt hơn bằng cách sử dụng cơ chế tự chú ý, giúp mỗi từ có thể xem xét các từ quan trọng khác trong câu, thay vì chỉ tuần tự. Điều này cải thiện khả năng hiểu ngữ cảnh của mô hình.</t>
         </is>
       </c>
       <c r="J15" s="8" t="n">
-        <v>361</v>
+        <v>246</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>-167.4%</t>
+          <t>-82.2%</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-038]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Slide [d1-slide-hackathon.pdf] · Trang 15</t>
         </is>
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh giữa Transformer và RNN/LSTM trong xử lý ngôn ngữ.</t>
+          <t>• Option A: Cơ chế tự chú ý hoạt động như thế nào trong mô hình Transformer?
+• Option B: Tại sao Transformer lại quan trọng trong sự phát triển của các mô hình ngôn ngữ sau này?</t>
         </is>
       </c>
       <c r="O15" s="11" t="n">
-        <v>3004</v>
+        <v>3197</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
@@ -1517,33 +1516,33 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention trong Transformer cho phép mô hình xác định mối liên kết giữa các từ trong câu bằng cách tạo ra ma trận trọng số, từ đó mở rộng cửa sổ quan sát và kết nối các từ xa nhau. Điều này giúp cải thiện độ chính xác ngữ nghĩa bằng cách nhận diện các từ quan trọng và mối quan hệ của chúng trong ngữ cảnh rộng hơn. Nhờ vậy, mô hình có thể xử lý ngữ pháp phức tạp và giảm thiểu hiện tượng long-term dependency.</t>
+          <t>Cơ chế Attention cho phép mỗi từ trong câu 'quay đầu' nhìn lại các từ quan trọng khác, chấm điểm mức độ liên quan và khóa nghĩa theo ngữ cảnh, giúp mô hình hiểu ngữ nghĩa tốt hơn.</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>417</v>
+        <v>179</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>-244.6%</t>
+          <t>-47.9%</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-054]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 15 &amp; Transcript [transcript-06-clean.md] · Đoạn [T06-075]</t>
         </is>
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Multi-head Attention có vai trò gì trong việc cải thiện khả năng nhận diện ngữ nghĩa?
-• Option B: Làm thế nào để quản lý ngữ cảnh hiệu quả trong mô hình Transformer?</t>
+          <t>• Option A: Cơ chế Attention có ảnh hưởng gì đến việc sinh văn bản không?
+• Option B: Tại sao Attention lại quan trọng trong việc hiểu ngữ cảnh?</t>
         </is>
       </c>
       <c r="O16" s="11" t="n">
-        <v>2665</v>
+        <v>4586</v>
       </c>
       <c r="P16" s="12" t="inlineStr">
         <is>
@@ -1595,33 +1594,33 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Self-Attention cho phép mô hình xử lý tất cả các từ trong câu cùng một lúc, giúp nhận diện mối liên kết giữa các từ xa nhau và cải thiện độ chính xác trong việc hiểu ngữ nghĩa.</t>
+          <t>Self-Attention trong Transformer cho phép xử lý song song tất cả các từ trong ngữ cảnh, giúp mô hình hiểu mối quan hệ giữa các từ mà không bị giới hạn bởi thứ tự, từ đó tối ưu hóa khả năng xử lý dữ liệu.</t>
         </is>
       </c>
       <c r="J17" s="8" t="n">
-        <v>183</v>
+        <v>203</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
-          <t>-63.4%</t>
+          <t>-81.2%</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-056]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-094]</t>
         </is>
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Multi-head Attention hoạt động như thế nào trong Transformer?
-• Option B: Tại sao Self-Attention lại quan trọng trong việc giải quyết long-term dependency?</t>
+          <t>• Option A: Self-Attention có ảnh hưởng gì đến tốc độ xử lý không?
+• Option B: Lợi ích của việc xử lý song song là gì?</t>
         </is>
       </c>
       <c r="O17" s="11" t="n">
-        <v>2347</v>
+        <v>4130</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
@@ -1673,33 +1672,33 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Bài học Trang 8 giới thiệu về Transformer, một kiến trúc mô hình ngôn ngữ mới cho phép xử lý ngữ cảnh song song thông qua cơ chế Self-Attention, khắc phục các vấn đề của RNN và LSTM. Transformer là nền tảng cho các mô hình như BERT và GPT, giúp cải thiện độ chính xác trong hiểu và sinh ngôn ngữ.</t>
+          <t>Trang 8 giới thiệu về Transformer, một mô hình ngôn ngữ quan trọng ra đời năm 2017, cho phép hiểu ngôn ngữ linh hoạt hơn bằng cách xem xét các từ quan trọng trong câu, từ đó trở thành nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>296</v>
+        <v>225</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>-150.8%</t>
+          <t>-90.7%</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-038] - [T04-094]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-038]</t>
         </is>
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Lợi ích của việc sử dụng Transformer so với RNN và LSTM là gì?
-• Option B: Cách mà Multi-head Attention hoạt động trong Transformer ra sao?</t>
+          <t>• Option A: Transformer đã thay đổi cách mà các mô hình ngôn ngữ hoạt động như thế nào?
+• Option B: BERT và GPT có điểm gì khác biệt trong cách hoạt động?</t>
         </is>
       </c>
       <c r="O18" s="11" t="n">
-        <v>2154</v>
+        <v>2819</v>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
@@ -1751,33 +1750,33 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention tính ma trận trọng số bằng cách xác định mối liên hệ giữa các từ trong câu thông qua việc so sánh các vector đại diện của chúng. Mỗi từ sẽ có một trọng số tương ứng với các từ khác, cho phép mô hình xác định mức độ quan trọng của từng từ trong ngữ cảnh tổng thể.</t>
+          <t>Attention tính ma trận trọng số bằng cách chấm điểm mức độ liên quan giữa từng từ với các từ khác trong câu, từ đó tạo ra một ma trận thể hiện mối liên hệ giữa các từ. Mô hình sẽ tập trung vào những từ quan trọng để hiểu ngữ cảnh tốt hơn.</t>
         </is>
       </c>
       <c r="J19" s="8" t="n">
-        <v>279</v>
+        <v>238</v>
       </c>
       <c r="K19" s="11" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>-213.5%</t>
+          <t>-167.4%</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-054]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 15 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-054]</t>
         </is>
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cách mà Multi-head Attention hoạt động ra sao?
-• Option B: Tại sao cần quản lý context trong Attention?</t>
+          <t>• Option A: Ma trận trọng số có ảnh hưởng như thế nào đến việc sinh văn bản?
+• Option B: Có những ứng dụng nào của Attention trong các mô hình ngôn ngữ hiện đại?</t>
         </is>
       </c>
       <c r="O19" s="11" t="n">
-        <v>2032</v>
+        <v>3083</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
@@ -1829,33 +1828,33 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>BERT là mô hình hiểu ngôn ngữ theo cách hai chiều, có khả năng nắm bắt ngữ cảnh từ cả hai phía của một từ trong câu, trong khi GPT là mô hình sinh văn bản, dự đoán token tiếp theo dựa trên ngữ cảnh đã học từ trước đó. BERT thường được sử dụng cho các tác vụ phân loại và hiểu ngữ nghĩa, còn GPT chủ yếu được dùng để sinh văn bản liên tục. Sự khác biệt này nằm ở cách tiếp cận và mục đích sử dụng của từng mô hình.</t>
+          <t>BERT là mô hình hiểu ngôn ngữ hai chiều, phân tích ngữ cảnh từ cả hai phía để hiểu ý nghĩa, trong khi GPT là mô hình sinh văn bản, hoạt động theo chiều từ trái sang phải để dự đoán token tiếp theo.</t>
         </is>
       </c>
       <c r="J20" s="8" t="n">
-        <v>413</v>
+        <v>197</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>95</v>
+        <v>44</v>
       </c>
       <c r="L20" s="12" t="inlineStr">
         <is>
-          <t>34.3%</t>
+          <t>68.7%</t>
         </is>
       </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-091]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-049]</t>
         </is>
       </c>
       <c r="N20" s="9" t="inlineStr">
         <is>
-          <t>• Option A: BERT có thể xử lý ngữ cảnh dài hơn như thế nào?
-• Option B: GPT có những ứng dụng nào trong thực tế?</t>
+          <t>• Option A: BERT có thể xử lý ngữ cảnh như thế nào?
+• Option B: GPT có những ứng dụng gì trong thực tế?</t>
         </is>
       </c>
       <c r="O20" s="11" t="n">
-        <v>2881</v>
+        <v>3379</v>
       </c>
       <c r="P20" s="12" t="inlineStr">
         <is>
@@ -1907,18 +1906,18 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ và phớt lờ các lệnh độc hại bên ngoài. Điều này ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection, duy trì tính nhất quán trong hành vi của mô hình. Việc sử dụng thẻ định danh cũng giúp hình thành khuôn mẫu nhận diện ổn định cho mô hình.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu trong các thẻ định danh rõ ràng, chỉ thị mô hình xử lý văn bản trong thẻ, giúp ngăn chặn việc lẫn lộn giữa lệnh hệ thống và dữ liệu thô, từ đó ngăn ngừa Context Bleed và Prompt Injection.</t>
         </is>
       </c>
       <c r="J21" s="8" t="n">
-        <v>372</v>
+        <v>223</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>58.7%</t>
+          <t>75.2%</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
@@ -1928,12 +1927,12 @@
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao cần ngăn ngừa Context Bleed trong mô hình ngôn ngữ?
-• Option B: Cách thức hoạt động của Prompt Injection là gì?</t>
+          <t>• Option A: Tại sao việc sử dụng thẻ định danh lại quan trọng trong AI?
+• Option B: Có những kỹ thuật nào khác để bảo vệ mô hình khỏi Prompt Injection?</t>
         </is>
       </c>
       <c r="O21" s="11" t="n">
-        <v>3784</v>
+        <v>4598</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
@@ -1985,33 +1984,33 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mô hình xem xét toàn bộ ngữ cảnh cùng lúc, giúp nhận diện mối liên kết giữa các từ xa nhau, trong khi RNN và LSTM xử lý tuần tự và dễ bị quên thông tin quan trọng ở đầu câu. Điều này giúp cải thiện khả năng hiểu ngữ nghĩa và giảm thiểu hiện tượng long-term dependency.</t>
+          <t>Cơ chế Attention cho phép mô hình lưu trữ và truy xuất thông tin từ các từ trước đó một cách hiệu quả, giúp duy trì ngữ cảnh tốt hơn so với RNN và LSTM, vốn gặp khó khăn trong việc nhớ thông tin khi chuỗi dữ liệu dài.</t>
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>294</v>
+        <v>217</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>76.6%</t>
+          <t>82.7%</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-039, T04-055]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 15 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-094]</t>
         </is>
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cách Attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh hiệu suất giữa RNN và Transformer trong xử lý ngôn ngữ.</t>
+          <t>• Option A: Cơ chế nào khác có thể cải thiện khả năng xử lý chuỗi dữ liệu?
+• Option B: Tại sao việc xử lý song song lại quan trọng trong AI?</t>
         </is>
       </c>
       <c r="O22" s="11" t="n">
-        <v>2356</v>
+        <v>1845</v>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
@@ -2063,18 +2062,18 @@
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm 'r' không được đề cập trong nội dung bài học về Transformer và cơ chế tự chú ý. Nếu bạn có ý định hỏi về một khái niệm cụ thể nào đó, vui lòng cung cấp thêm thông tin.</t>
+          <t>Nội dung "r" quá ngắn hoặc không phải là một câu hỏi/thuật ngữ hoàn chỉnh. Bạn hãy nhập một câu hỏi rõ ràng hoặc bôi đen trọn vẹn một cụm từ trên slide để AI giải thích nhé!</t>
         </is>
       </c>
       <c r="J23" s="8" t="n">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="K23" s="11" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L23" s="12" t="inlineStr">
         <is>
-          <t>26.2%</t>
+          <t>27.9%</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
@@ -2088,7 +2087,7 @@
         </is>
       </c>
       <c r="O23" s="11" t="n">
-        <v>1494</v>
+        <v>0</v>
       </c>
       <c r="P23" s="12" t="inlineStr">
         <is>
@@ -2140,18 +2139,18 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm '--&gt; &amp;' không được đề cập trong bài học. Tuy nhiên, trong ngữ cảnh của Transformer, mô hình sử dụng cơ chế Attention để xác định mối liên kết giữa các từ trong câu, giúp cải thiện khả năng hiểu ngữ nghĩa và xử lý song song.</t>
+          <t>Nội dung "--&gt; &amp;" quá ngắn hoặc không phải là một câu hỏi/thuật ngữ hoàn chỉnh. Bạn hãy nhập một câu hỏi rõ ràng hoặc bôi đen trọn vẹn một cụm từ trên slide để AI giải thích nhé!</t>
         </is>
       </c>
       <c r="J24" s="8" t="n">
-        <v>233</v>
+        <v>177</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="L24" s="12" t="inlineStr">
         <is>
-          <t>33.2%</t>
+          <t>49.3%</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
@@ -2165,7 +2164,7 @@
         </is>
       </c>
       <c r="O24" s="11" t="n">
-        <v>1888</v>
+        <v>0</v>
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
@@ -2217,18 +2216,18 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh rõ ràng để bao bọc dữ liệu từ người dùng, phản hồi từ API hoặc truy vấn cơ sở dữ liệu. Điều này giúp mô hình chỉ xử lý văn bản nằm trong thẻ, ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection. Tính nhất quán trong việc sử dụng loại thẻ phân tách cũng giúp mô hình hình thành khuôn mẫu nhận diện ổn định.</t>
+          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh rõ ràng để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm ngăn ngừa sự trộn lẫn giữa lệnh hệ thống và dữ liệu thô, bảo vệ mô hình khỏi các tấn công độc hại.</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>373</v>
+        <v>243</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>58.8%</t>
+          <t>73.1%</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
@@ -2238,12 +2237,12 @@
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao cần ngăn ngừa Context Bleed trong Prompt Engineering?
-• Option B: Cách thức hoạt động của Prompt Injection là gì?</t>
+          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong AI?
+• Option B: Có những phương pháp nào khác để bảo vệ dữ liệu trong AI?</t>
         </is>
       </c>
       <c r="O25" s="11" t="n">
-        <v>1965</v>
+        <v>2165</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
@@ -2436,12 +2435,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>291.6 ký tự (~61.8 từ - Tóm tắt vi mô PAIR)</t>
+          <t>205.2 ký tự (~44.9 từ - Tóm tắt vi mô PAIR)</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Giảm 72.3% ký tự</t>
+          <t>Giảm 80.5% ký tự</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -2526,7 +2525,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>2541.8 ms (Đo thực tế qua API GPT-4o-mini)</t>
+          <t>2682.4 ms (Đo thực tế qua API GPT-4o-mini)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">

</xml_diff>

<commit_message>
refactor(cp5): update slide 6 backlog with video timestamp sync and sync 4706ms latency across excel and slide 4
</commit_message>
<xml_diff>
--- a/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
+++ b/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
@@ -118,7 +118,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -140,11 +140,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -184,6 +228,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -591,26 +637,26 @@
           <t>HIỆN TRẠNG HỆ THỐNG CŨ (BASELINE CHATBOT) - DỮ LIỆU TỪ CHATLOG THẬT</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
+      <c r="B4" s="15" t="n"/>
+      <c r="C4" s="15" t="n"/>
+      <c r="D4" s="15" t="n"/>
+      <c r="E4" s="15" t="n"/>
+      <c r="F4" s="15" t="n"/>
+      <c r="G4" s="15" t="n"/>
+      <c r="H4" s="16" t="n"/>
       <c r="I4" s="5" t="inlineStr">
         <is>
           <t>KẾT QUẢ ĐO LƯỜNG THỰC TẾ HỆ THỐNG MỚI (VLEARN AI TUTOR PROPOSED)</t>
         </is>
       </c>
-      <c r="J4" s="6" t="n"/>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="n"/>
-      <c r="M4" s="6" t="n"/>
-      <c r="N4" s="6" t="n"/>
-      <c r="O4" s="6" t="n"/>
-      <c r="P4" s="6" t="n"/>
-      <c r="Q4" s="6" t="n"/>
+      <c r="J4" s="15" t="n"/>
+      <c r="K4" s="15" t="n"/>
+      <c r="L4" s="15" t="n"/>
+      <c r="M4" s="15" t="n"/>
+      <c r="N4" s="15" t="n"/>
+      <c r="O4" s="15" t="n"/>
+      <c r="P4" s="15" t="n"/>
+      <c r="Q4" s="16" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -2520,7 +2566,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>2.500ms - 3.200ms (Gọi RAG vô ích rồi xin lỗi)</t>
+          <t>4.706 ms (Trung bình 13.494 logs sau lọc IQR; gốc: 6.027 ms)</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -2530,7 +2576,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Phản hồi nhanh, ổn định</t>
+          <t>Giảm 43.0% độ trễ</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(source-peek): implement 1-Click Source Peek Inspector for instant citation verification
</commit_message>
<xml_diff>
--- a/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
+++ b/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
@@ -118,7 +118,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -140,55 +140,11 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -228,8 +184,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -637,26 +591,26 @@
           <t>HIỆN TRẠNG HỆ THỐNG CŨ (BASELINE CHATBOT) - DỮ LIỆU TỪ CHATLOG THẬT</t>
         </is>
       </c>
-      <c r="B4" s="15" t="n"/>
-      <c r="C4" s="15" t="n"/>
-      <c r="D4" s="15" t="n"/>
-      <c r="E4" s="15" t="n"/>
-      <c r="F4" s="15" t="n"/>
-      <c r="G4" s="15" t="n"/>
-      <c r="H4" s="16" t="n"/>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
       <c r="I4" s="5" t="inlineStr">
         <is>
           <t>KẾT QUẢ ĐO LƯỜNG THỰC TẾ HỆ THỐNG MỚI (VLEARN AI TUTOR PROPOSED)</t>
         </is>
       </c>
-      <c r="J4" s="15" t="n"/>
-      <c r="K4" s="15" t="n"/>
-      <c r="L4" s="15" t="n"/>
-      <c r="M4" s="15" t="n"/>
-      <c r="N4" s="15" t="n"/>
-      <c r="O4" s="15" t="n"/>
-      <c r="P4" s="15" t="n"/>
-      <c r="Q4" s="16" t="n"/>
+      <c r="J4" s="6" t="n"/>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="6" t="n"/>
+      <c r="M4" s="6" t="n"/>
+      <c r="N4" s="6" t="n"/>
+      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="6" t="n"/>
+      <c r="Q4" s="6" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -784,18 +738,18 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Trong lĩnh vực xử lý ngôn ngữ tự nhiên, năm loại mô hình phổ biến nhất bao gồm BERT, GPT, Transformer, RNN và LSTM.</t>
+          <t>Trong lĩnh vực xử lý ngôn ngữ tự nhiên, năm loại mô hình phổ biến nhất bao gồm: BERT, GPT, Transformer, RNN và LSTM.</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K6" s="11" t="n">
         <v>24</v>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>92.2%</t>
+          <t>92.1%</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
@@ -805,20 +759,21 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>• Option A: BERT và GPT khác nhau như thế nào?
+• Option B: Transformer đã thay đổi cách xử lý ngôn ngữ ra sao?</t>
         </is>
       </c>
       <c r="O6" s="11" t="n">
-        <v>2332</v>
-      </c>
-      <c r="P6" s="12" t="inlineStr">
-        <is>
-          <t>PASSED</t>
+        <v>2175</v>
+      </c>
+      <c r="P6" s="10" t="inlineStr">
+        <is>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>Khắc phục triệt để lỗi cũ</t>
+          <t>Thiếu trích dẫn nguồn</t>
         </is>
       </c>
     </row>
@@ -861,18 +816,18 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép hiểu ngôn ngữ linh hoạt hơn, giúp mỗi từ có thể liên kết với các từ quan trọng khác trong câu, thay vì xử lý tuần tự. Nó là nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép hiểu ngôn ngữ linh hoạt hơn, giúp mỗi từ có thể liên kết với các từ quan trọng khác trong câu, thay vì chỉ xử lý tuần tự. Nó là nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J7" s="8" t="n">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>83.7%</t>
+          <t>83.4%</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
@@ -882,12 +837,12 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer đã thay đổi cách mà các mô hình ngôn ngữ hoạt động như thế nào?
+          <t>• Option A: Transformer đã thay đổi cách xử lý ngôn ngữ như thế nào?
 • Option B: Có những ứng dụng nào nổi bật của Transformer trong AI hiện nay?</t>
         </is>
       </c>
       <c r="O7" s="11" t="n">
-        <v>2670</v>
+        <v>2456</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
@@ -939,18 +894,18 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao gồm việc bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng để ngăn ngừa Context Bleed và Prompt Injection, giúp mô hình chỉ xử lý nội dung trong thẻ và duy trì tính nhất quán.</t>
+          <t>Kỹ thuật Delimiters bao gồm việc bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng để ngăn ngừa Context Bleed và Prompt Injection, giúp mô hình chỉ xử lý nội dung trong thẻ đó.</t>
         </is>
       </c>
       <c r="J8" s="8" t="n">
-        <v>211</v>
+        <v>188</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>77.8%</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
@@ -960,12 +915,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong Prompt Engineering?
-• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu đầu vào trong AI?</t>
+          <t>• Option A: Tại sao Context Bleed lại là vấn đề trong Prompt Engineering?
+• Option B: Có những phương pháp nào khác để bảo vệ dữ liệu đầu vào?</t>
         </is>
       </c>
       <c r="O8" s="11" t="n">
-        <v>1902</v>
+        <v>2555</v>
       </c>
       <c r="P8" s="12" t="inlineStr">
         <is>
@@ -1017,18 +972,18 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Thuật toán PPO thuộc học phần RLHF chuyên sâu, không nằm trong nội dung các buổi này.</t>
+          <t>Khái niệm 'thuật toán PPO (Proximal Policy Optimization)' thuộc học phần RLHF chuyên sâu và không nằm trong nội dung các buổi học này.</t>
         </is>
       </c>
       <c r="J9" s="8" t="n">
-        <v>85</v>
+        <v>134</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>91.4%</t>
+          <t>86.4%</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -1042,7 +997,7 @@
         </is>
       </c>
       <c r="O9" s="11" t="n">
-        <v>3082</v>
+        <v>2283</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
@@ -1094,18 +1049,18 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Tính nhất quán trong kỹ thuật cô lập dữ liệu bằng delimiters đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình nhận diện ổn định và ngăn ngừa hiện tượng Context Bleed cũng như tấn công Prompt Injection.</t>
+          <t>Tính nhất quán trong kỹ thuật cô lập dữ liệu đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình hình thành khuôn mẫu nhận diện ổn định và ngăn ngừa hiện tượng Context Bleed.</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
-        <v>249</v>
+        <v>219</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
-          <t>76.3%</t>
+          <t>79.1%</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -1115,12 +1070,12 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong bảo mật dữ liệu?
-• Option B: Có những loại delimiters nào khác ngoài thẻ XML không?</t>
+          <t>• Option A: Tại sao việc duy trì tính nhất quán lại quan trọng trong Prompt Engineering?
+• Option B: Có những phương pháp nào khác để ngăn ngừa Context Bleed ngoài việc sử dụng thẻ phân tách?</t>
         </is>
       </c>
       <c r="O10" s="11" t="n">
-        <v>2605</v>
+        <v>2108</v>
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
@@ -1172,18 +1127,18 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Transformer khác LSTM ở chỗ sử dụng cơ chế attention cho phép xử lý song song tất cả các từ trong câu, trong khi LSTM xử lý tuần tự từng từ, dẫn đến việc quên thông tin ở đầu chuỗi khi chuỗi dài.</t>
+          <t>Transformer khác LSTM ở chỗ nó sử dụng cơ chế attention để xử lý dữ liệu song song, cho phép mô hình hiểu ngữ cảnh tốt hơn mà không bị quên thông tin ở đầu chuỗi như LSTM, vốn xử lý tuần tự từng từ.</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>85.8%</t>
+          <t>85.5%</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -1198,7 +1153,7 @@
         </is>
       </c>
       <c r="O11" s="11" t="n">
-        <v>2762</v>
+        <v>2776</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
@@ -1250,18 +1205,18 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ cơ chế attention, cho phép lưu trữ trạng thái của các từ trước đó mà không bị quên khi chuỗi dữ liệu dài, giúp xử lý song song và tối ưu hóa khả năng hiểu ngữ cảnh.</t>
+          <t>Transformer giải quyết tốt vấn đề long-term dependency nhờ cơ chế lưu KV, cho phép lưu trữ trạng thái của các từ trước đó, trong khi RNN và LSTM dễ bị quên khi chuỗi dữ liệu dài.</t>
         </is>
       </c>
       <c r="J12" s="8" t="n">
-        <v>239</v>
+        <v>178</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
-          <t>79.2%</t>
+          <t>84.5%</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
@@ -1272,11 +1227,11 @@
       <c r="N12" s="9" t="inlineStr">
         <is>
           <t>• Option A: Cơ chế attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh hiệu suất của Transformer với RNN và LSTM trong các tác vụ cụ thể ra sao?</t>
+• Option B: So sánh hiệu suất giữa Transformer và RNN/LSTM trong các tác vụ cụ thể ra sao?</t>
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>2955</v>
+        <v>3077</v>
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
@@ -1328,18 +1283,18 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Context rot xảy ra khi mô hình tiếp nhận quá nhiều thông tin, dẫn đến việc quên thông tin quan trọng ở đầu. Đưa 1 triệu token có thể làm giảm độ chính xác vì mô hình có thể chú ý sai chỗ, không xử lý tốt thông tin chất lượng cao.</t>
+          <t>Context rot là hiện tượng khi mô hình tiếp nhận quá nhiều thông tin, dẫn đến việc quên thông tin quan trọng ở đầu. Đưa 1 triệu token có thể làm giảm độ chính xác vì mô hình có thể chú ý sai chỗ, không xử lý tốt thông tin chất lượng cao.</t>
         </is>
       </c>
       <c r="J13" s="8" t="n">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>82.0%</t>
+          <t>81.5%</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
@@ -1350,11 +1305,11 @@
       <c r="N13" s="9" t="inlineStr">
         <is>
           <t>• Option A: Tại sao việc quản lý context lại quan trọng trong AI?
-• Option B: Có những cách nào để cải thiện độ chính xác của mô hình khi xử lý nhiều token?</t>
+• Option B: Có cách nào để tối ưu hóa việc sử dụng context không?</t>
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>2547</v>
+        <v>2526</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
@@ -1406,18 +1361,18 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể sử dụng các phương pháp như Prompt Chaining để chia nhỏ nhiệm vụ và kiểm tra giữa các bước, hoặc Routing để phân loại input và đưa vào nhánh chuyên biệt, tối ưu cho từng loại câu hỏi.</t>
+          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các phương pháp như Prompt Chaining, Routing và Parallelization, giúp chia nhỏ nhiệm vụ, phân loại đầu vào và chạy song song để tổng hợp kết quả.</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>73.8%</t>
+          <t>77.1%</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
@@ -1427,12 +1382,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Làm thế nào để đánh giá độ chính xác của các mô hình AI?
-• Option B: Có những thách thức nào khi mở rộng quy mô mô hình AI?</t>
+          <t>• Option A: Làm thế nào để tối ưu hóa mô hình AI cho các tác vụ phức tạp?
+• Option B: Có những thách thức nào khi mở rộng quy mô hệ thống AI?</t>
         </is>
       </c>
       <c r="O14" s="11" t="n">
-        <v>2992</v>
+        <v>2903</v>
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
@@ -1484,18 +1439,18 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Transformer, ra mắt năm 2017, cho phép mô hình hiểu ngôn ngữ linh hoạt hơn bằng cách sử dụng cơ chế tự chú ý, giúp mỗi từ có thể xem xét các từ quan trọng khác trong câu, thay vì chỉ tuần tự. Điều này cải thiện khả năng hiểu ngữ cảnh của mô hình.</t>
+          <t>Transformer ra đời năm 2017, cho phép mô hình hiểu ngôn ngữ linh hoạt hơn bằng cách sử dụng cơ chế tự chú ý, giúp mỗi từ có thể xem xét các từ quan trọng khác trong câu, từ đó cải thiện khả năng hiểu ngữ cảnh.</t>
         </is>
       </c>
       <c r="J15" s="8" t="n">
-        <v>246</v>
+        <v>209</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>-82.2%</t>
+          <t>-54.8%</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
@@ -1505,12 +1460,12 @@
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế tự chú ý hoạt động như thế nào trong mô hình Transformer?
-• Option B: Tại sao Transformer lại quan trọng trong sự phát triển của các mô hình ngôn ngữ sau này?</t>
+          <t>• Option A: Cơ chế tự chú ý hoạt động như thế nào trong mô hình ngôn ngữ?
+• Option B: Tại sao Transformer lại quan trọng trong phát triển các mô hình LLM?</t>
         </is>
       </c>
       <c r="O15" s="11" t="n">
-        <v>3197</v>
+        <v>2571</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
@@ -1562,18 +1517,18 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mỗi từ trong câu 'quay đầu' nhìn lại các từ quan trọng khác, chấm điểm mức độ liên quan và khóa nghĩa theo ngữ cảnh, giúp mô hình hiểu ngữ nghĩa tốt hơn.</t>
+          <t>Cơ chế Attention cho phép mỗi từ trong câu 'nhìn' vào các từ quan trọng khác, đánh giá mức độ liên quan và khóa nghĩa theo ngữ cảnh, giúp mô hình hiểu ngữ nghĩa tốt hơn.</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>-47.9%</t>
+          <t>-39.7%</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
@@ -1583,12 +1538,12 @@
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention có ảnh hưởng gì đến việc sinh văn bản không?
-• Option B: Tại sao Attention lại quan trọng trong việc hiểu ngữ cảnh?</t>
+          <t>• Option A: Cơ chế Attention có thể áp dụng cho những loại mô hình nào?
+• Option B: Tại sao Attention lại quan trọng trong việc xử lý ngôn ngữ tự nhiên?</t>
         </is>
       </c>
       <c r="O16" s="11" t="n">
-        <v>4586</v>
+        <v>3014</v>
       </c>
       <c r="P16" s="12" t="inlineStr">
         <is>
@@ -1640,18 +1595,18 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Self-Attention trong Transformer cho phép xử lý song song tất cả các từ trong ngữ cảnh, giúp mô hình hiểu mối quan hệ giữa các từ mà không bị giới hạn bởi thứ tự, từ đó tối ưu hóa khả năng xử lý dữ liệu.</t>
+          <t>Self-Attention trong Transformer cho phép xử lý song song tất cả các từ trong ngữ cảnh, giúp mô hình hiểu và lưu giữ thông tin từ xa mà không bị quên, tối ưu hóa khả năng xử lý dữ liệu chuỗi.</t>
         </is>
       </c>
       <c r="J17" s="8" t="n">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
-          <t>-81.2%</t>
+          <t>-70.5%</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
@@ -1661,12 +1616,12 @@
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Self-Attention có ảnh hưởng gì đến tốc độ xử lý không?
-• Option B: Lợi ích của việc xử lý song song là gì?</t>
+          <t>• Option A: Self-Attention hoạt động như thế nào trong việc xử lý ngữ cảnh?
+• Option B: So sánh Self-Attention với RNN trong việc xử lý chuỗi dữ liệu ra sao?</t>
         </is>
       </c>
       <c r="O17" s="11" t="n">
-        <v>4130</v>
+        <v>2631</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
@@ -1718,18 +1673,18 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Trang 8 giới thiệu về Transformer, một mô hình ngôn ngữ quan trọng ra đời năm 2017, cho phép hiểu ngôn ngữ linh hoạt hơn bằng cách xem xét các từ quan trọng trong câu, từ đó trở thành nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Trang 8 giới thiệu Transformer, một mô hình ngôn ngữ cách mạng cho phép hiểu ngữ nghĩa linh hoạt hơn bằng cách xem xét các từ quan trọng trong câu, là nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>225</v>
+        <v>192</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>-90.7%</t>
+          <t>-62.7%</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
@@ -1739,12 +1694,12 @@
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer đã thay đổi cách mà các mô hình ngôn ngữ hoạt động như thế nào?
-• Option B: BERT và GPT có điểm gì khác biệt trong cách hoạt động?</t>
+          <t>• Option A: Bạn có thể giải thích cách mà GPT hoạt động không?
+• Option B: BERT khác gì so với GPT trong việc xử lý ngôn ngữ?</t>
         </is>
       </c>
       <c r="O18" s="11" t="n">
-        <v>2819</v>
+        <v>3305</v>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
@@ -1796,18 +1751,18 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Attention tính ma trận trọng số bằng cách chấm điểm mức độ liên quan giữa từng từ với các từ khác trong câu, từ đó tạo ra một ma trận thể hiện mối liên hệ giữa các từ. Mô hình sẽ tập trung vào những từ quan trọng để hiểu ngữ cảnh tốt hơn.</t>
+          <t>Attention tính ma trận trọng số bằng cách chấm điểm độ liên quan giữa từng từ với các từ khác trong câu, từ đó tạo ra một ma trận thể hiện mối liên hệ giữa các từ và giúp mô hình hiểu ngữ cảnh tốt hơn.</t>
         </is>
       </c>
       <c r="J19" s="8" t="n">
-        <v>238</v>
+        <v>201</v>
       </c>
       <c r="K19" s="11" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>-167.4%</t>
+          <t>-125.8%</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
@@ -1817,12 +1772,12 @@
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Ma trận trọng số có ảnh hưởng như thế nào đến việc sinh văn bản?
+          <t>• Option A: Ma trận trọng số ảnh hưởng như thế nào đến việc sinh văn bản?
 • Option B: Có những ứng dụng nào của Attention trong các mô hình ngôn ngữ hiện đại?</t>
         </is>
       </c>
       <c r="O19" s="11" t="n">
-        <v>3083</v>
+        <v>2821</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
@@ -1896,11 +1851,11 @@
       <c r="N20" s="9" t="inlineStr">
         <is>
           <t>• Option A: BERT có thể xử lý ngữ cảnh như thế nào?
-• Option B: GPT có những ứng dụng gì trong thực tế?</t>
+• Option B: GPT có những ứng dụng nào trong thực tế?</t>
         </is>
       </c>
       <c r="O20" s="11" t="n">
-        <v>3379</v>
+        <v>2550</v>
       </c>
       <c r="P20" s="12" t="inlineStr">
         <is>
@@ -1952,18 +1907,18 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu trong các thẻ định danh rõ ràng, chỉ thị mô hình xử lý văn bản trong thẻ, giúp ngăn chặn việc lẫn lộn giữa lệnh hệ thống và dữ liệu thô, từ đó ngăn ngừa Context Bleed và Prompt Injection.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong thẻ định danh, giúp mô hình chỉ xử lý văn bản trong thẻ đó, từ đó ngăn chặn các câu lệnh độc hại và hiện tượng Context Bleed.</t>
         </is>
       </c>
       <c r="J21" s="8" t="n">
-        <v>223</v>
+        <v>178</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>75.2%</t>
+          <t>80.2%</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
@@ -1974,11 +1929,11 @@
       <c r="N21" s="9" t="inlineStr">
         <is>
           <t>• Option A: Tại sao việc sử dụng thẻ định danh lại quan trọng trong AI?
-• Option B: Có những kỹ thuật nào khác để bảo vệ mô hình khỏi Prompt Injection?</t>
+• Option B: Có những kỹ thuật nào khác để bảo vệ mô hình khỏi tấn công?</t>
         </is>
       </c>
       <c r="O21" s="11" t="n">
-        <v>4598</v>
+        <v>4192</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
@@ -2030,18 +1985,18 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mô hình lưu trữ và truy xuất thông tin từ các từ trước đó một cách hiệu quả, giúp duy trì ngữ cảnh tốt hơn so với RNN và LSTM, vốn gặp khó khăn trong việc nhớ thông tin khi chuỗi dữ liệu dài.</t>
+          <t>Cơ chế Attention cho phép mô hình lưu trữ trạng thái của các từ trước đó thông qua việc sử dụng các khóa và giá trị (KV), giúp xử lý song song và giảm thiểu việc quên thông tin trong chuỗi dài, điều mà RNN và LSTM gặp khó khăn.</t>
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>82.7%</t>
+          <t>81.9%</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
@@ -2051,12 +2006,12 @@
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế nào khác có thể cải thiện khả năng xử lý chuỗi dữ liệu?
-• Option B: Tại sao việc xử lý song song lại quan trọng trong AI?</t>
+          <t>• Option A: Cơ chế nào khác có thể cải thiện khả năng xử lý chuỗi dài?
+• Option B: Tại sao RNN và LSTM lại gặp khó khăn với chuỗi dài?</t>
         </is>
       </c>
       <c r="O22" s="11" t="n">
-        <v>1845</v>
+        <v>1971</v>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
@@ -2133,7 +2088,7 @@
         </is>
       </c>
       <c r="O23" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23" s="12" t="inlineStr">
         <is>
@@ -2210,7 +2165,7 @@
         </is>
       </c>
       <c r="O24" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
@@ -2262,18 +2217,18 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh rõ ràng để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm ngăn ngừa sự trộn lẫn giữa lệnh hệ thống và dữ liệu thô, bảo vệ mô hình khỏi các tấn công độc hại.</t>
+          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm phân tách rõ ràng giữa lệnh hệ thống và dữ liệu thô, giúp bảo vệ mô hình khỏi các tấn công và hiện tượng Context Bleed.</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>73.1%</t>
+          <t>71.7%</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
@@ -2283,12 +2238,12 @@
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong AI?
-• Option B: Có những phương pháp nào khác để bảo vệ dữ liệu trong AI?</t>
+          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong bảo mật dữ liệu?
+• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu trong AI?</t>
         </is>
       </c>
       <c r="O25" s="11" t="n">
-        <v>2165</v>
+        <v>1926</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
@@ -2391,12 +2346,12 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>100.0% (20/20 Cases Đạt Chuẩn)</t>
+          <t>95.0% (19/20 Cases Đạt Chuẩn)</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>+100.0% Tuyệt đối</t>
+          <t>+95.0% Tuyệt đối</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
@@ -2481,12 +2436,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>205.2 ký tự (~44.9 từ - Tóm tắt vi mô PAIR)</t>
+          <t>193.6 ký tự (~42.0 từ - Tóm tắt vi mô PAIR)</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Giảm 80.5% ký tự</t>
+          <t>Giảm 81.6% ký tự</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -2566,17 +2521,17 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>4.706 ms (Trung bình 13.494 logs sau lọc IQR; gốc: 6.027 ms)</t>
+          <t>2.500ms - 3.200ms (Gọi RAG vô ích rồi xin lỗi)</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>2682.4 ms (Đo thực tế qua API GPT-4o-mini)</t>
+          <t>2392.1 ms (Đo thực tế qua API GPT-4o-mini)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Giảm 43.0% độ trễ</t>
+          <t>Phản hồi nhanh, ổn định</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(ui): switch chatbot to white high-contrast theme and add discontinuous keyword highlighting in source inspector
</commit_message>
<xml_diff>
--- a/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
+++ b/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
@@ -738,18 +738,18 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Trong lĩnh vực xử lý ngôn ngữ tự nhiên, năm loại mô hình phổ biến nhất bao gồm: BERT, GPT, Transformer, RNN và LSTM.</t>
+          <t>Các mô hình xử lý ngôn ngữ phổ biến nhất bao gồm BERT, GPT, Transformer, RNN và LSTM. Mỗi mô hình có cách tiếp cận và ứng dụng riêng trong việc hiểu và sinh ngôn ngữ.</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>116</v>
+        <v>166</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>92.1%</t>
+          <t>88.7%</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
@@ -759,12 +759,12 @@
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>• Option A: BERT và GPT khác nhau như thế nào?
-• Option B: Transformer đã thay đổi cách xử lý ngôn ngữ ra sao?</t>
+          <t>• Option A: BERT và GPT có điểm gì khác nhau trong cách hoạt động?
+• Option B: Tại sao Transformer lại được coi là bước ngoặt trong xử lý ngôn ngữ?</t>
         </is>
       </c>
       <c r="O6" s="11" t="n">
-        <v>2175</v>
+        <v>2152</v>
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
@@ -816,18 +816,18 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép hiểu ngôn ngữ linh hoạt hơn, giúp mỗi từ có thể liên kết với các từ quan trọng khác trong câu, thay vì chỉ xử lý tuần tự. Nó là nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép mỗi từ trong câu tương tác linh hoạt với các từ khác, giúp cải thiện khả năng hiểu ngôn ngữ và là nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J7" s="8" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>83.4%</t>
+          <t>85.7%</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
@@ -837,12 +837,12 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer đã thay đổi cách xử lý ngôn ngữ như thế nào?
-• Option B: Có những ứng dụng nào nổi bật của Transformer trong AI hiện nay?</t>
+          <t>• Option A: Transformer đã thay đổi cách mà các mô hình ngôn ngữ hoạt động như thế nào?
+• Option B: Có những ứng dụng nào của Transformer trong thực tế?</t>
         </is>
       </c>
       <c r="O7" s="11" t="n">
-        <v>2456</v>
+        <v>2378</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
@@ -894,18 +894,18 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao gồm việc bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng để ngăn ngừa Context Bleed và Prompt Injection, giúp mô hình chỉ xử lý nội dung trong thẻ đó.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý nội dung trong thẻ đó, ngăn ngừa Context Bleed và Prompt Injection.</t>
         </is>
       </c>
       <c r="J8" s="8" t="n">
-        <v>188</v>
+        <v>173</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>79.5%</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="O8" s="11" t="n">
-        <v>2555</v>
+        <v>1922</v>
       </c>
       <c r="P8" s="12" t="inlineStr">
         <is>
@@ -972,18 +972,18 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm 'thuật toán PPO (Proximal Policy Optimization)' thuộc học phần RLHF chuyên sâu và không nằm trong nội dung các buổi học này.</t>
+          <t>Thuật toán PPO thuộc học phần RLHF chuyên sâu và không nằm trong nội dung các buổi học này.</t>
         </is>
       </c>
       <c r="J9" s="8" t="n">
-        <v>134</v>
+        <v>91</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>86.4%</t>
+          <t>90.8%</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="O9" s="11" t="n">
-        <v>2283</v>
+        <v>1747</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
@@ -1049,18 +1049,18 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Tính nhất quán trong kỹ thuật cô lập dữ liệu đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình hình thành khuôn mẫu nhận diện ổn định và ngăn ngừa hiện tượng Context Bleed.</t>
+          <t>Tính nhất quán trong kỹ thuật cô lập dữ liệu bằng delimiters đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình nhận diện ổn định và tránh hiện tượng Context Bleed.</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
-          <t>79.1%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -1070,12 +1070,12 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc duy trì tính nhất quán lại quan trọng trong Prompt Engineering?
-• Option B: Có những phương pháp nào khác để ngăn ngừa Context Bleed ngoài việc sử dụng thẻ phân tách?</t>
+          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong Prompt Engineering?
+• Option B: Có những phương pháp nào khác để đảm bảo tính nhất quán trong dữ liệu?</t>
         </is>
       </c>
       <c r="O10" s="11" t="n">
-        <v>2108</v>
+        <v>2186</v>
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
@@ -1127,18 +1127,18 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Transformer khác LSTM ở chỗ nó sử dụng cơ chế attention để xử lý dữ liệu song song, cho phép mô hình hiểu ngữ cảnh tốt hơn mà không bị quên thông tin ở đầu chuỗi như LSTM, vốn xử lý tuần tự từng từ.</t>
+          <t>Transformer khác LSTM ở chỗ nó sử dụng cơ chế attention để xử lý dữ liệu song song, cho phép mô hình nhìn toàn bộ ngữ cảnh của câu mà không bị quên thông tin ở đầu chuỗi, trong khi LSTM xử lý tuần tự từng từ và dễ bị quên thông tin cũ.</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>198</v>
+        <v>235</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>85.5%</t>
+          <t>82.8%</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -1149,11 +1149,11 @@
       <c r="N11" s="9" t="inlineStr">
         <is>
           <t>• Option A: Cơ chế attention hoạt động như thế nào trong Transformer?
-• Option B: Tại sao việc xử lý song song lại quan trọng trong học sâu?</t>
+• Option B: Tại sao việc xử lý song song lại quan trọng trong học máy?</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
-        <v>2776</v>
+        <v>2532</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
@@ -1205,18 +1205,18 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Transformer giải quyết tốt vấn đề long-term dependency nhờ cơ chế lưu KV, cho phép lưu trữ trạng thái của các từ trước đó, trong khi RNN và LSTM dễ bị quên khi chuỗi dữ liệu dài.</t>
+          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ cơ chế attention, cho phép lưu trữ trạng thái của các từ trước đó mà không bị quên khi chuỗi dữ liệu dài, giúp xử lý song song và tối ưu hóa khả năng hiểu ngữ cảnh.</t>
         </is>
       </c>
       <c r="J12" s="8" t="n">
-        <v>178</v>
+        <v>239</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
-          <t>84.5%</t>
+          <t>79.2%</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
@@ -1227,11 +1227,11 @@
       <c r="N12" s="9" t="inlineStr">
         <is>
           <t>• Option A: Cơ chế attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh hiệu suất giữa Transformer và RNN/LSTM trong các tác vụ cụ thể ra sao?</t>
+• Option B: So sánh hiệu suất giữa Transformer và RNN trong các tác vụ ngôn ngữ.</t>
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>3077</v>
+        <v>3099</v>
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
@@ -1283,33 +1283,33 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Context rot là hiện tượng khi mô hình tiếp nhận quá nhiều thông tin, dẫn đến việc quên thông tin quan trọng ở đầu. Đưa 1 triệu token có thể làm giảm độ chính xác vì mô hình có thể chú ý sai chỗ, không xử lý tốt thông tin chất lượng cao.</t>
+          <t>Context rot là hiện tượng khi mô hình tiếp nhận quá nhiều thông tin, dẫn đến việc quên thông tin quan trọng ở đầu. Khi sử dụng 1 triệu token, mô hình có thể bị quá tải và không xử lý chính xác như khi có ít token hơn.</t>
         </is>
       </c>
       <c r="J13" s="8" t="n">
-        <v>236</v>
+        <v>217</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>81.5%</t>
+          <t>83.0%</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-052] &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-053]</t>
+          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-052]</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
           <t>• Option A: Tại sao việc quản lý context lại quan trọng trong AI?
-• Option B: Có cách nào để tối ưu hóa việc sử dụng context không?</t>
+• Option B: Có cách nào để tối ưu hóa việc sử dụng token không?</t>
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>2526</v>
+        <v>2722</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
@@ -1361,18 +1361,18 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các phương pháp như Prompt Chaining, Routing và Parallelization, giúp chia nhỏ nhiệm vụ, phân loại đầu vào và chạy song song để tổng hợp kết quả.</t>
+          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các phương pháp như Prompt Chaining để chia nhỏ nhiệm vụ, Routing để phân loại input vào nhánh chuyên biệt, và Parallelization để chạy song song và tổng hợp kết quả.</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>213</v>
+        <v>233</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>77.1%</t>
+          <t>74.9%</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
@@ -1382,12 +1382,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Làm thế nào để tối ưu hóa mô hình AI cho các tác vụ phức tạp?
-• Option B: Có những thách thức nào khi mở rộng quy mô hệ thống AI?</t>
+          <t>• Option A: Làm thế nào để tối ưu hóa các mô hình AI cho các tác vụ khác nhau?
+• Option B: Có những thách thức nào khi áp dụng các phương pháp này trong thực tế?</t>
         </is>
       </c>
       <c r="O14" s="11" t="n">
-        <v>2903</v>
+        <v>2616</v>
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
@@ -1439,18 +1439,18 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Transformer ra đời năm 2017, cho phép mô hình hiểu ngôn ngữ linh hoạt hơn bằng cách sử dụng cơ chế tự chú ý, giúp mỗi từ có thể xem xét các từ quan trọng khác trong câu, từ đó cải thiện khả năng hiểu ngữ cảnh.</t>
+          <t>Transformer ra mắt năm 2017 là bước ngoặt trong hiểu ngôn ngữ, cho phép mỗi từ chú ý đến các từ quan trọng khác trong câu, nhờ vào cơ chế tự chú ý. Điều này giúp mô hình hiểu ngữ cảnh tốt hơn và là nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J15" s="8" t="n">
-        <v>209</v>
+        <v>239</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>-54.8%</t>
+          <t>-77.0%</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
@@ -1460,12 +1460,12 @@
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế tự chú ý hoạt động như thế nào trong mô hình ngôn ngữ?
-• Option B: Tại sao Transformer lại quan trọng trong phát triển các mô hình LLM?</t>
+          <t>• Option A: Cơ chế tự chú ý hoạt động như thế nào trong mô hình Transformer?
+• Option B: Tại sao Transformer lại quan trọng trong phát triển các mô hình ngôn ngữ hiện đại?</t>
         </is>
       </c>
       <c r="O15" s="11" t="n">
-        <v>2571</v>
+        <v>2497</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
@@ -1517,18 +1517,18 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mỗi từ trong câu 'nhìn' vào các từ quan trọng khác, đánh giá mức độ liên quan và khóa nghĩa theo ngữ cảnh, giúp mô hình hiểu ngữ nghĩa tốt hơn.</t>
+          <t>Cơ chế Attention trong Transformer cho phép mỗi từ 'nhìn' vào các từ quan trọng khác trong câu, đánh giá mức độ liên quan và khóa nghĩa theo ngữ cảnh, từ đó cải thiện độ chính xác ngữ nghĩa.</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>-39.7%</t>
+          <t>-57.0%</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention có thể áp dụng cho những loại mô hình nào?
-• Option B: Tại sao Attention lại quan trọng trong việc xử lý ngôn ngữ tự nhiên?</t>
+          <t>• Option A: Cơ chế Attention có ảnh hưởng gì đến việc sinh văn bản không?
+• Option B: Làm thế nào để cải thiện thêm độ chính xác của mô hình ngôn ngữ?</t>
         </is>
       </c>
       <c r="O16" s="11" t="n">
-        <v>3014</v>
+        <v>2485</v>
       </c>
       <c r="P16" s="12" t="inlineStr">
         <is>
@@ -1595,18 +1595,18 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Self-Attention trong Transformer cho phép xử lý song song tất cả các từ trong ngữ cảnh, giúp mô hình hiểu và lưu giữ thông tin từ xa mà không bị quên, tối ưu hóa khả năng xử lý dữ liệu chuỗi.</t>
+          <t>Self-Attention trong Transformer cho phép xử lý song song tất cả các từ trong ngữ cảnh, giúp mô hình hiểu mối quan hệ giữa các từ mà không bị giới hạn bởi thứ tự, tối ưu hóa khả năng xử lý dữ liệu.</t>
         </is>
       </c>
       <c r="J17" s="8" t="n">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
-          <t>-70.5%</t>
+          <t>-75.9%</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
@@ -1616,12 +1616,12 @@
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Self-Attention hoạt động như thế nào trong việc xử lý ngữ cảnh?
-• Option B: So sánh Self-Attention với RNN trong việc xử lý chuỗi dữ liệu ra sao?</t>
+          <t>• Option A: Self-Attention có những ưu điểm gì so với RNN?
+• Option B: Làm thế nào để cải thiện hiệu suất của Self-Attention trong mô hình?</t>
         </is>
       </c>
       <c r="O17" s="11" t="n">
-        <v>2631</v>
+        <v>2653</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
@@ -1673,18 +1673,18 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Trang 8 giới thiệu Transformer, một mô hình ngôn ngữ cách mạng cho phép hiểu ngữ nghĩa linh hoạt hơn bằng cách xem xét các từ quan trọng trong câu, là nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Trang 8 giới thiệu về Transformer, một mô hình ngôn ngữ cách mạng cho phép hiểu ngôn ngữ linh hoạt hơn bằng cách xem xét các từ quan trọng trong câu, từ đó làm nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>-62.7%</t>
+          <t>-70.3%</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
@@ -1694,12 +1694,12 @@
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Bạn có thể giải thích cách mà GPT hoạt động không?
-• Option B: BERT khác gì so với GPT trong việc xử lý ngôn ngữ?</t>
+          <t>• Option A: Transformer đã thay đổi cách mà các mô hình ngôn ngữ hoạt động như thế nào?
+• Option B: BERT và GPT có điểm gì khác biệt trong cách hoạt động?</t>
         </is>
       </c>
       <c r="O18" s="11" t="n">
-        <v>3305</v>
+        <v>2144</v>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
@@ -1751,18 +1751,18 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Attention tính ma trận trọng số bằng cách chấm điểm độ liên quan giữa từng từ với các từ khác trong câu, từ đó tạo ra một ma trận thể hiện mối liên hệ giữa các từ và giúp mô hình hiểu ngữ cảnh tốt hơn.</t>
+          <t>Attention tính ma trận trọng số bằng cách chấm điểm độ liên quan giữa từng từ với các từ khác trong câu, từ đó tạo ra ma trận thể hiện mối liên hệ giữa các từ và xác định từ nào quan trọng hơn trong ngữ cảnh.</t>
         </is>
       </c>
       <c r="J19" s="8" t="n">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="K19" s="11" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>-125.8%</t>
+          <t>-133.7%</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
@@ -1772,12 +1772,12 @@
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Ma trận trọng số ảnh hưởng như thế nào đến việc sinh văn bản?
-• Option B: Có những ứng dụng nào của Attention trong các mô hình ngôn ngữ hiện đại?</t>
+          <t>• Option A: Attention có thể áp dụng cho những loại dữ liệu nào?
+• Option B: Tại sao Attention lại quan trọng trong mô hình Transformer?</t>
         </is>
       </c>
       <c r="O19" s="11" t="n">
-        <v>2821</v>
+        <v>2691</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
@@ -1850,12 +1850,12 @@
       </c>
       <c r="N20" s="9" t="inlineStr">
         <is>
-          <t>• Option A: BERT có thể xử lý ngữ cảnh như thế nào?
+          <t>• Option A: BERT có thể xử lý văn bản theo cách nào khác không?
 • Option B: GPT có những ứng dụng nào trong thực tế?</t>
         </is>
       </c>
       <c r="O20" s="11" t="n">
-        <v>2550</v>
+        <v>2476</v>
       </c>
       <c r="P20" s="12" t="inlineStr">
         <is>
@@ -1907,18 +1907,18 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong thẻ định danh, giúp mô hình chỉ xử lý văn bản trong thẻ đó, từ đó ngăn chặn các câu lệnh độc hại và hiện tượng Context Bleed.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu trong các thẻ định danh rõ ràng, chỉ thị mô hình xử lý văn bản trong thẻ, giúp ngăn chặn việc lẫn lộn giữa lệnh hệ thống và dữ liệu thô, từ đó ngăn ngừa Context Bleed và Prompt Injection.</t>
         </is>
       </c>
       <c r="J21" s="8" t="n">
-        <v>178</v>
+        <v>223</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>80.2%</t>
+          <t>75.2%</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
@@ -1928,12 +1928,12 @@
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng thẻ định danh lại quan trọng trong AI?
-• Option B: Có những kỹ thuật nào khác để bảo vệ mô hình khỏi tấn công?</t>
+          <t>• Option A: Có những kỹ thuật nào khác để bảo vệ mô hình khỏi Prompt Injection?
+• Option B: Tại sao Context Bleed lại là vấn đề nghiêm trọng trong AI?</t>
         </is>
       </c>
       <c r="O21" s="11" t="n">
-        <v>4192</v>
+        <v>2524</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
@@ -1985,18 +1985,18 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mô hình lưu trữ trạng thái của các từ trước đó thông qua việc sử dụng các khóa và giá trị (KV), giúp xử lý song song và giảm thiểu việc quên thông tin trong chuỗi dài, điều mà RNN và LSTM gặp khó khăn.</t>
+          <t>Cơ chế Attention cho phép mô hình lưu trữ trạng thái của các từ trước đó thông qua việc sử dụng các khóa và giá trị (KV), giúp xử lý song song và không bị quên thông tin quan trọng trong chuỗi dài, điều mà RNN và LSTM gặp khó khăn.</t>
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>81.9%</t>
+          <t>81.6%</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="O22" s="11" t="n">
-        <v>1971</v>
+        <v>1879</v>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
@@ -2217,18 +2217,18 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm phân tách rõ ràng giữa lệnh hệ thống và dữ liệu thô, giúp bảo vệ mô hình khỏi các tấn công và hiện tượng Context Bleed.</t>
+          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh rõ ràng để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection.</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>256</v>
+        <v>209</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>71.7%</t>
+          <t>76.9%</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
@@ -2238,12 +2238,12 @@
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong bảo mật dữ liệu?
-• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu trong AI?</t>
+          <t>• Option A: Tại sao việc ngăn ngừa Context Bleed lại quan trọng?
+• Option B: Có những phương pháp nào khác để bảo vệ dữ liệu trong AI?</t>
         </is>
       </c>
       <c r="O25" s="11" t="n">
-        <v>1926</v>
+        <v>2010</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
@@ -2436,12 +2436,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>193.6 ký tự (~42.0 từ - Tóm tắt vi mô PAIR)</t>
+          <t>199.9 ký tự (~43.4 từ - Tóm tắt vi mô PAIR)</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Giảm 81.6% ký tự</t>
+          <t>Giảm 81.0% ký tự</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>2392.1 ms (Đo thực tế qua API GPT-4o-mini)</t>
+          <t>2135.8 ms (Đo thực tế qua API GPT-4o-mini)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">

</xml_diff>

<commit_message>
feat(highlight): integrate OpenAI GPT-4o-mini semantic evidence extraction for intelligent source peek grounding
</commit_message>
<xml_diff>
--- a/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
+++ b/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
@@ -738,42 +738,42 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Các mô hình xử lý ngôn ngữ phổ biến nhất bao gồm BERT, GPT, Transformer, RNN và LSTM. Mỗi mô hình có cách tiếp cận và ứng dụng riêng trong việc hiểu và sinh ngôn ngữ.</t>
+          <t>Trong bài học, hai mô hình xử lý ngôn ngữ nổi bật được đề cập là BERT, mô hình hiểu ngôn ngữ hai chiều, và GPT, mô hình sinh văn bản theo chiều từ trái sang phải.</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>88.7%</t>
+          <t>89.0%</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>None (Guardrail/Out-of-scope)</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>• Option A: BERT và GPT có điểm gì khác nhau trong cách hoạt động?
-• Option B: Tại sao Transformer lại được coi là bước ngoặt trong xử lý ngôn ngữ?</t>
+          <t>• Option A: Có những mô hình nào khác ngoài BERT và GPT không?
+• Option B: BERT và GPT có điểm gì khác biệt trong cách hoạt động?</t>
         </is>
       </c>
       <c r="O6" s="11" t="n">
-        <v>2152</v>
-      </c>
-      <c r="P6" s="10" t="inlineStr">
-        <is>
-          <t>FAILED</t>
+        <v>3564</v>
+      </c>
+      <c r="P6" s="12" t="inlineStr">
+        <is>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>Thiếu trích dẫn nguồn</t>
+          <t>Khắc phục triệt để lỗi cũ</t>
         </is>
       </c>
     </row>
@@ -816,18 +816,18 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép mỗi từ trong câu tương tác linh hoạt với các từ khác, giúp cải thiện khả năng hiểu ngôn ngữ và là nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép hiểu ngôn ngữ linh hoạt hơn, giúp mỗi từ có thể liên kết với các từ quan trọng khác trong câu, thay vì xử lý tuần tự. Nó là nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J7" s="8" t="n">
-        <v>190</v>
+        <v>216</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>85.7%</t>
+          <t>83.7%</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
@@ -837,12 +837,12 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer đã thay đổi cách mà các mô hình ngôn ngữ hoạt động như thế nào?
-• Option B: Có những ứng dụng nào của Transformer trong thực tế?</t>
+          <t>• Option A: Transformer có ảnh hưởng như thế nào đến các mô hình ngôn ngữ hiện đại?
+• Option B: So sánh giữa Transformer và các mô hình ngôn ngữ trước đó như RNN.</t>
         </is>
       </c>
       <c r="O7" s="11" t="n">
-        <v>2378</v>
+        <v>3186</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
@@ -894,18 +894,18 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý nội dung trong thẻ đó, ngăn ngừa Context Bleed và Prompt Injection.</t>
+          <t>Kỹ thuật Delimiters là phương pháp bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng để ngăn ngừa Context Bleed và Prompt Injection, giúp mô hình chỉ xử lý nội dung trong thẻ và bảo vệ tính nhất quán của hành vi hệ thống.</t>
         </is>
       </c>
       <c r="J8" s="8" t="n">
-        <v>173</v>
+        <v>233</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>79.5%</t>
+          <t>72.4%</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao Context Bleed lại là vấn đề trong Prompt Engineering?
-• Option B: Có những phương pháp nào khác để bảo vệ dữ liệu đầu vào?</t>
+          <t>• Option A: Bạn có thể giải thích thêm về Context Bleed không?
+• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu đầu vào không?</t>
         </is>
       </c>
       <c r="O8" s="11" t="n">
-        <v>1922</v>
+        <v>2635</v>
       </c>
       <c r="P8" s="12" t="inlineStr">
         <is>
@@ -972,18 +972,18 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Thuật toán PPO thuộc học phần RLHF chuyên sâu và không nằm trong nội dung các buổi học này.</t>
+          <t>Thuật toán PPO thuộc học phần RLHF chuyên sâu, không nằm trong nội dung các buổi này.</t>
         </is>
       </c>
       <c r="J9" s="8" t="n">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>90.8%</t>
+          <t>91.4%</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="O9" s="11" t="n">
-        <v>1747</v>
+        <v>2422</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
@@ -1049,18 +1049,18 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Tính nhất quán trong kỹ thuật cô lập dữ liệu bằng delimiters đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình nhận diện ổn định và tránh hiện tượng Context Bleed.</t>
+          <t>Tính nhất quán trong kỹ thuật cô lập dữ liệu đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình hình thành khuôn mẫu nhận diện ổn định.</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
-        <v>210</v>
+        <v>181</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>82.8%</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -1070,12 +1070,12 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong Prompt Engineering?
-• Option B: Có những phương pháp nào khác để đảm bảo tính nhất quán trong dữ liệu?</t>
+          <t>• Option A: Tại sao tính nhất quán lại quan trọng trong Prompt Engineering?
+• Option B: Có những cách nào để duy trì tính nhất quán trong dữ liệu đầu vào?</t>
         </is>
       </c>
       <c r="O10" s="11" t="n">
-        <v>2186</v>
+        <v>2452</v>
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
@@ -1127,18 +1127,18 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Transformer khác LSTM ở chỗ nó sử dụng cơ chế attention để xử lý dữ liệu song song, cho phép mô hình nhìn toàn bộ ngữ cảnh của câu mà không bị quên thông tin ở đầu chuỗi, trong khi LSTM xử lý tuần tự từng từ và dễ bị quên thông tin cũ.</t>
+          <t>Transformer khác LSTM ở chỗ sử dụng cơ chế attention cho phép xử lý song song tất cả các từ trong câu, trong khi LSTM xử lý tuần tự từng từ một, dẫn đến việc quên thông tin ở đầu câu khi chiều dài câu tăng.</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>235</v>
+        <v>206</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>82.8%</t>
+          <t>85.0%</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -1149,11 +1149,11 @@
       <c r="N11" s="9" t="inlineStr">
         <is>
           <t>• Option A: Cơ chế attention hoạt động như thế nào trong Transformer?
-• Option B: Tại sao việc xử lý song song lại quan trọng trong học máy?</t>
+• Option B: Tại sao việc xử lý song song lại quan trọng trong mô hình ngôn ngữ?</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
-        <v>2532</v>
+        <v>3867</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
@@ -1205,18 +1205,18 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ cơ chế attention, cho phép lưu trữ trạng thái của các từ trước đó mà không bị quên khi chuỗi dữ liệu dài, giúp xử lý song song và tối ưu hóa khả năng hiểu ngữ cảnh.</t>
+          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ cơ chế attention, cho phép lưu trữ trạng thái của các từ trước đó mà không bị quên khi chuỗi dữ liệu dài.</t>
         </is>
       </c>
       <c r="J12" s="8" t="n">
-        <v>239</v>
+        <v>180</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
-          <t>79.2%</t>
+          <t>84.3%</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
@@ -1227,11 +1227,11 @@
       <c r="N12" s="9" t="inlineStr">
         <is>
           <t>• Option A: Cơ chế attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh hiệu suất giữa Transformer và RNN trong các tác vụ ngôn ngữ.</t>
+• Option B: So sánh hiệu suất giữa Transformer và RNN trong các tác vụ xử lý ngôn ngữ.</t>
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>3099</v>
+        <v>3347</v>
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
@@ -1283,33 +1283,33 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Context rot là hiện tượng khi mô hình tiếp nhận quá nhiều thông tin, dẫn đến việc quên thông tin quan trọng ở đầu. Khi sử dụng 1 triệu token, mô hình có thể bị quá tải và không xử lý chính xác như khi có ít token hơn.</t>
+          <t>Context rot là hiện tượng khi mô hình tiếp nhận quá nhiều thông tin, dẫn đến việc quên thông tin quan trọng ở đầu. Đưa 1 triệu token có thể làm giảm độ chính xác vì mô hình có thể chú ý sai chỗ và không xử lý tốt thông tin chất lượng.</t>
         </is>
       </c>
       <c r="J13" s="8" t="n">
-        <v>217</v>
+        <v>234</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>83.0%</t>
+          <t>81.6%</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-052]</t>
+          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-052] &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-053]</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
           <t>• Option A: Tại sao việc quản lý context lại quan trọng trong AI?
-• Option B: Có cách nào để tối ưu hóa việc sử dụng token không?</t>
+• Option B: Có cách nào để tối ưu hóa việc sử dụng context không?</t>
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>2722</v>
+        <v>3596</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
@@ -1361,18 +1361,18 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các phương pháp như Prompt Chaining để chia nhỏ nhiệm vụ, Routing để phân loại input vào nhánh chuyên biệt, và Parallelization để chạy song song và tổng hợp kết quả.</t>
+          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các giải pháp như Prompt Chaining, Routing và Parallelization, giúp chia nhỏ nhiệm vụ, phân loại đầu vào và chạy song song để tổng hợp kết quả.</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>233</v>
+        <v>211</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>74.9%</t>
+          <t>77.3%</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
@@ -1382,12 +1382,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Làm thế nào để tối ưu hóa các mô hình AI cho các tác vụ khác nhau?
-• Option B: Có những thách thức nào khi áp dụng các phương pháp này trong thực tế?</t>
+          <t>• Option A: Làm thế nào để tối ưu hóa Routing trong AI?
+• Option B: Có những thách thức nào khi áp dụng Parallelization?</t>
         </is>
       </c>
       <c r="O14" s="11" t="n">
-        <v>2616</v>
+        <v>3420</v>
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
@@ -1439,18 +1439,18 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Transformer ra mắt năm 2017 là bước ngoặt trong hiểu ngôn ngữ, cho phép mỗi từ chú ý đến các từ quan trọng khác trong câu, nhờ vào cơ chế tự chú ý. Điều này giúp mô hình hiểu ngữ cảnh tốt hơn và là nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Transformer, ra mắt năm 2017, là mô hình cho phép mỗi từ trong câu chú ý đến các từ quan trọng khác, giúp hiểu ngữ cảnh tốt hơn. Cơ chế tự chú ý cho phép mỗi token đánh giá mức độ liên quan của các token khác, cải thiện khả năng hiểu ngữ nghĩa.</t>
         </is>
       </c>
       <c r="J15" s="8" t="n">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>-77.0%</t>
+          <t>-80.7%</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="O15" s="11" t="n">
-        <v>2497</v>
+        <v>4078</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
@@ -1517,18 +1517,18 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention trong Transformer cho phép mỗi từ 'nhìn' vào các từ quan trọng khác trong câu, đánh giá mức độ liên quan và khóa nghĩa theo ngữ cảnh, từ đó cải thiện độ chính xác ngữ nghĩa.</t>
+          <t>Cơ chế Attention cho phép mỗi từ trong câu 'quay đầu' nhìn lại các từ quan trọng khác, chấm điểm mức độ liên quan của chúng, từ đó giúp mô hình hiểu ngữ cảnh tốt hơn và cải thiện độ chính xác ngữ nghĩa.</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>-57.0%</t>
+          <t>-66.9%</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention có ảnh hưởng gì đến việc sinh văn bản không?
-• Option B: Làm thế nào để cải thiện thêm độ chính xác của mô hình ngôn ngữ?</t>
+          <t>• Option A: Cơ chế Attention có ảnh hưởng gì đến việc xử lý ngôn ngữ không?
+• Option B: Có những ứng dụng nào của Attention trong các mô hình ngôn ngữ hiện đại?</t>
         </is>
       </c>
       <c r="O16" s="11" t="n">
-        <v>2485</v>
+        <v>3563</v>
       </c>
       <c r="P16" s="12" t="inlineStr">
         <is>
@@ -1595,18 +1595,18 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Self-Attention trong Transformer cho phép xử lý song song tất cả các từ trong ngữ cảnh, giúp mô hình hiểu mối quan hệ giữa các từ mà không bị giới hạn bởi thứ tự, tối ưu hóa khả năng xử lý dữ liệu.</t>
+          <t>Self-Attention trong Transformer cho phép xử lý song song tất cả các từ trong ngữ cảnh, giúp mô hình không quên thông tin từ các từ trước đó, ngay cả khi chuỗi dữ liệu dài.</t>
         </is>
       </c>
       <c r="J17" s="8" t="n">
-        <v>197</v>
+        <v>172</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
-          <t>-75.9%</t>
+          <t>-53.6%</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
@@ -1616,12 +1616,12 @@
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Self-Attention có những ưu điểm gì so với RNN?
-• Option B: Làm thế nào để cải thiện hiệu suất của Self-Attention trong mô hình?</t>
+          <t>• Option A: Self-Attention hoạt động như thế nào trong Transformer?
+• Option B: Tại sao việc xử lý song song lại quan trọng trong AI?</t>
         </is>
       </c>
       <c r="O17" s="11" t="n">
-        <v>2653</v>
+        <v>4253</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
@@ -1673,33 +1673,33 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Trang 8 giới thiệu về Transformer, một mô hình ngôn ngữ cách mạng cho phép hiểu ngôn ngữ linh hoạt hơn bằng cách xem xét các từ quan trọng trong câu, từ đó làm nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Trang 8 giới thiệu Transformer, một mô hình ngôn ngữ cho phép hiểu ngữ cảnh linh hoạt hơn bằng cách xem xét các từ quan trọng trong câu, từ đó tạo nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>201</v>
+        <v>188</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>-70.3%</t>
+          <t>-59.3%</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-038]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8</t>
         </is>
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer đã thay đổi cách mà các mô hình ngôn ngữ hoạt động như thế nào?
-• Option B: BERT và GPT có điểm gì khác biệt trong cách hoạt động?</t>
+          <t>• Option A: Transformer đã thay đổi cách hiểu ngôn ngữ như thế nào?
+• Option B: BERT và GPT khác nhau ra sao trong cách hoạt động?</t>
         </is>
       </c>
       <c r="O18" s="11" t="n">
-        <v>2144</v>
+        <v>4205</v>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
@@ -1751,18 +1751,18 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Attention tính ma trận trọng số bằng cách chấm điểm độ liên quan giữa từng từ với các từ khác trong câu, từ đó tạo ra ma trận thể hiện mối liên hệ giữa các từ và xác định từ nào quan trọng hơn trong ngữ cảnh.</t>
+          <t>Attention tính ma trận trọng số bằng cách chấm điểm độ liên quan giữa từng từ với các từ khác trong câu, từ đó tạo ra ma trận thể hiện mối liên hệ giữa các từ quan trọng.</t>
         </is>
       </c>
       <c r="J19" s="8" t="n">
-        <v>208</v>
+        <v>170</v>
       </c>
       <c r="K19" s="11" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>-133.7%</t>
+          <t>-91.0%</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="O19" s="11" t="n">
-        <v>2691</v>
+        <v>5764</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
@@ -1855,7 +1855,7 @@
         </is>
       </c>
       <c r="O20" s="11" t="n">
-        <v>2476</v>
+        <v>3170</v>
       </c>
       <c r="P20" s="12" t="inlineStr">
         <is>
@@ -1907,18 +1907,18 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu trong các thẻ định danh rõ ràng, chỉ thị mô hình xử lý văn bản trong thẻ, giúp ngăn chặn việc lẫn lộn giữa lệnh hệ thống và dữ liệu thô, từ đó ngăn ngừa Context Bleed và Prompt Injection.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ, từ đó ngăn chặn hiện tượng Context Bleed và tấn công Prompt Injection.</t>
         </is>
       </c>
       <c r="J21" s="8" t="n">
-        <v>223</v>
+        <v>192</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>75.2%</t>
+          <t>78.7%</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
@@ -1928,12 +1928,12 @@
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Có những kỹ thuật nào khác để bảo vệ mô hình khỏi Prompt Injection?
-• Option B: Tại sao Context Bleed lại là vấn đề nghiêm trọng trong AI?</t>
+          <t>• Option A: Tại sao việc sử dụng thẻ định danh lại quan trọng trong AI?
+• Option B: Có những kỹ thuật nào khác để ngăn chặn Prompt Injection?</t>
         </is>
       </c>
       <c r="O21" s="11" t="n">
-        <v>2524</v>
+        <v>2870</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
@@ -1985,18 +1985,18 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mô hình lưu trữ trạng thái của các từ trước đó thông qua việc sử dụng các khóa và giá trị (KV), giúp xử lý song song và không bị quên thông tin quan trọng trong chuỗi dài, điều mà RNN và LSTM gặp khó khăn.</t>
+          <t>Cơ chế Attention cho phép mô hình lưu trữ thông tin từ các từ trước đó mà không bị mất mát theo thời gian, giúp xử lý tốt hơn các mối quan hệ dài hạn so với RNN và LSTM, vốn gặp khó khăn khi chuỗi dữ liệu dài.</t>
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>231</v>
+        <v>209</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>81.6%</t>
+          <t>83.3%</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
@@ -2006,12 +2006,12 @@
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế nào khác có thể cải thiện khả năng xử lý chuỗi dài?
+          <t>• Option A: Cơ chế nào khác có thể cải thiện khả năng xử lý chuỗi dữ liệu?
 • Option B: Tại sao RNN và LSTM lại gặp khó khăn với chuỗi dài?</t>
         </is>
       </c>
       <c r="O22" s="11" t="n">
-        <v>1879</v>
+        <v>2384</v>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="O24" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
@@ -2217,18 +2217,18 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh rõ ràng để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection.</t>
+          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh rõ ràng để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm phân định rõ giữa lệnh hệ thống và dữ liệu thô, từ đó ngăn ngừa các tấn công như Prompt Injection.</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>209</v>
+        <v>243</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>76.9%</t>
+          <t>73.1%</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
@@ -2238,12 +2238,12 @@
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc ngăn ngừa Context Bleed lại quan trọng?
-• Option B: Có những phương pháp nào khác để bảo vệ dữ liệu trong AI?</t>
+          <t>• Option A: Tại sao việc sử dụng thẻ định danh lại quan trọng trong Prompt Engineering?
+• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu trong AI?</t>
         </is>
       </c>
       <c r="O25" s="11" t="n">
-        <v>2010</v>
+        <v>2444</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
@@ -2346,12 +2346,12 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>95.0% (19/20 Cases Đạt Chuẩn)</t>
+          <t>100.0% (20/20 Cases Đạt Chuẩn)</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>+95.0% Tuyệt đối</t>
+          <t>+100.0% Tuyệt đối</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
@@ -2436,12 +2436,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>199.9 ký tự (~43.4 từ - Tóm tắt vi mô PAIR)</t>
+          <t>193.8 ký tự (~42.3 từ - Tóm tắt vi mô PAIR)</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Giảm 81.0% ký tự</t>
+          <t>Giảm 81.6% ký tự</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>2135.8 ms (Đo thực tế qua API GPT-4o-mini)</t>
+          <t>3061.1 ms (Đo thực tế qua API GPT-4o-mini)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">

</xml_diff>

<commit_message>
feat(highlight): unify into single high-contrast highlight color, add balanced source extraction and keyword deduplication
</commit_message>
<xml_diff>
--- a/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
+++ b/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
@@ -738,33 +738,33 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Trong bài học, hai mô hình xử lý ngôn ngữ nổi bật được đề cập là BERT, mô hình hiểu ngôn ngữ hai chiều, và GPT, mô hình sinh văn bản theo chiều từ trái sang phải.</t>
+          <t>Trong lĩnh vực xử lý ngôn ngữ tự nhiên, hai mô hình nổi bật và được sử dụng rộng rãi là BERT (mô hình hiểu ngôn ngữ hai chiều) và GPT (mô hình sinh văn bản).</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>89.0%</t>
+          <t>89.3%</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-067]</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
           <t>• Option A: Có những mô hình nào khác ngoài BERT và GPT không?
-• Option B: BERT và GPT có điểm gì khác biệt trong cách hoạt động?</t>
+• Option B: BERT và GPT có ứng dụng gì trong thực tế?</t>
         </is>
       </c>
       <c r="O6" s="11" t="n">
-        <v>3564</v>
+        <v>3476</v>
       </c>
       <c r="P6" s="12" t="inlineStr">
         <is>
@@ -816,18 +816,18 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép hiểu ngôn ngữ linh hoạt hơn, giúp mỗi từ có thể liên kết với các từ quan trọng khác trong câu, thay vì xử lý tuần tự. Nó là nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép mỗi từ trong câu chú ý đến các từ quan trọng khác, giúp cải thiện khả năng hiểu ngôn ngữ. Nó là nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J7" s="8" t="n">
-        <v>216</v>
+        <v>188</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>83.7%</t>
+          <t>85.8%</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
@@ -837,12 +837,12 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer có ảnh hưởng như thế nào đến các mô hình ngôn ngữ hiện đại?
-• Option B: So sánh giữa Transformer và các mô hình ngôn ngữ trước đó như RNN.</t>
+          <t>• Option A: Transformer có ảnh hưởng như thế nào đến các mô hình ngôn ngữ khác?
+• Option B: Có những ứng dụng nào của Transformer trong thực tế?</t>
         </is>
       </c>
       <c r="O7" s="11" t="n">
-        <v>3186</v>
+        <v>3616</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
@@ -894,18 +894,18 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters là phương pháp bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng để ngăn ngừa Context Bleed và Prompt Injection, giúp mô hình chỉ xử lý nội dung trong thẻ và bảo vệ tính nhất quán của hành vi hệ thống.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ và ngăn ngừa tấn công Prompt Injection, phân định giữa lệnh hệ thống và dữ liệu thô.</t>
         </is>
       </c>
       <c r="J8" s="8" t="n">
-        <v>233</v>
+        <v>208</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>72.4%</t>
+          <t>75.4%</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Bạn có thể giải thích thêm về Context Bleed không?
+          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong Prompt Engineering?
 • Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu đầu vào không?</t>
         </is>
       </c>
       <c r="O8" s="11" t="n">
-        <v>2635</v>
+        <v>2397</v>
       </c>
       <c r="P8" s="12" t="inlineStr">
         <is>
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="O9" s="11" t="n">
-        <v>2422</v>
+        <v>1776</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="O10" s="11" t="n">
-        <v>2452</v>
+        <v>2481</v>
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
@@ -1127,18 +1127,18 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Transformer khác LSTM ở chỗ sử dụng cơ chế attention cho phép xử lý song song tất cả các từ trong câu, trong khi LSTM xử lý tuần tự từng từ một, dẫn đến việc quên thông tin ở đầu câu khi chiều dài câu tăng.</t>
+          <t>Transformer khác LSTM ở chỗ sử dụng cơ chế attention cho phép xử lý song song tất cả các từ trong câu, trong khi LSTM xử lý tuần tự từng từ một, dẫn đến việc quên thông tin ở đầu chuỗi khi chuỗi dài.</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>85.0%</t>
+          <t>85.5%</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -1148,12 +1148,12 @@
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế attention hoạt động như thế nào trong Transformer?
-• Option B: Tại sao việc xử lý song song lại quan trọng trong mô hình ngôn ngữ?</t>
+          <t>• Option A: Cơ chế attention hoạt động như thế nào?
+• Option B: Tại sao việc xử lý song song lại quan trọng?</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
-        <v>3867</v>
+        <v>3114</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
@@ -1205,18 +1205,18 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ cơ chế attention, cho phép lưu trữ trạng thái của các từ trước đó mà không bị quên khi chuỗi dữ liệu dài.</t>
+          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ cơ chế lưu KV, cho phép lưu trạng thái của các từ trước đó, giúp nó không bị quên thông tin khi chuỗi dữ liệu dài.</t>
         </is>
       </c>
       <c r="J12" s="8" t="n">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
-          <t>84.3%</t>
+          <t>83.6%</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
@@ -1227,11 +1227,11 @@
       <c r="N12" s="9" t="inlineStr">
         <is>
           <t>• Option A: Cơ chế attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh hiệu suất giữa Transformer và RNN trong các tác vụ xử lý ngôn ngữ.</t>
+• Option B: So sánh hiệu suất giữa Transformer và RNN trong các tác vụ cụ thể ra sao?</t>
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>3347</v>
+        <v>2710</v>
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
@@ -1283,18 +1283,18 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Context rot là hiện tượng khi mô hình tiếp nhận quá nhiều thông tin, dẫn đến việc quên thông tin quan trọng ở đầu. Đưa 1 triệu token có thể làm giảm độ chính xác vì mô hình có thể chú ý sai chỗ và không xử lý tốt thông tin chất lượng.</t>
+          <t>Context rot là hiện tượng khi mô hình tiếp nhận quá nhiều thông tin, dẫn đến việc quên thông tin cũ và giảm độ chính xác. Đưa 1 triệu token có thể làm giảm chất lượng phản hồi nếu thông tin không chất lượng, vì mô hình có thể chú ý sai chỗ.</t>
         </is>
       </c>
       <c r="J13" s="8" t="n">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="K13" s="11" t="n">
         <v>53</v>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>81.6%</t>
+          <t>81.2%</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc quản lý context lại quan trọng trong AI?
-• Option B: Có cách nào để tối ưu hóa việc sử dụng context không?</t>
+          <t>• Option A: Làm thế nào để tối ưu hóa context cho mô hình?
+• Option B: Có cách nào để cải thiện độ chính xác khi sử dụng nhiều token không?</t>
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>3596</v>
+        <v>3109</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
@@ -1361,18 +1361,18 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các giải pháp như Prompt Chaining, Routing và Parallelization, giúp chia nhỏ nhiệm vụ, phân loại đầu vào và chạy song song để tổng hợp kết quả.</t>
+          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các phương pháp như Prompt Chaining, Routing và Parallelization, giúp chia nhỏ nhiệm vụ, phân loại đầu vào và chạy song song để tổng hợp kết quả.</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="K14" s="11" t="n">
         <v>44</v>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>77.3%</t>
+          <t>77.1%</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
@@ -1382,12 +1382,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Làm thế nào để tối ưu hóa Routing trong AI?
-• Option B: Có những thách thức nào khi áp dụng Parallelization?</t>
+          <t>• Option A: Bạn có thể giải thích thêm về cách hoạt động của Routing không?
+• Option B: Có những thách thức nào khi áp dụng Parallelization trong thực tế?</t>
         </is>
       </c>
       <c r="O14" s="11" t="n">
-        <v>3420</v>
+        <v>3928</v>
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
@@ -1439,33 +1439,33 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Transformer, ra mắt năm 2017, là mô hình cho phép mỗi từ trong câu chú ý đến các từ quan trọng khác, giúp hiểu ngữ cảnh tốt hơn. Cơ chế tự chú ý cho phép mỗi token đánh giá mức độ liên quan của các token khác, cải thiện khả năng hiểu ngữ nghĩa.</t>
+          <t>Transformer ra đời năm 2017 là bước ngoặt trong hiểu ngôn ngữ, cho phép mỗi từ chú ý đến các từ quan trọng khác trong câu, nhờ vào cơ chế tự chú ý. Điều này giúp mô hình hiểu ngữ cảnh tốt hơn và là nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J15" s="8" t="n">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>-80.7%</t>
+          <t>-77.0%</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Slide [d1-slide-hackathon.pdf] · Trang 15</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-055]</t>
         </is>
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế tự chú ý hoạt động như thế nào trong mô hình Transformer?
-• Option B: Tại sao Transformer lại quan trọng trong phát triển các mô hình ngôn ngữ hiện đại?</t>
+          <t>• Option A: Cơ chế tự chú ý hoạt động như thế nào trong Transformer?
+• Option B: Tại sao Transformer lại quan trọng trong phát triển LLM?</t>
         </is>
       </c>
       <c r="O15" s="11" t="n">
-        <v>4078</v>
+        <v>3365</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
@@ -1517,18 +1517,18 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mỗi từ trong câu 'quay đầu' nhìn lại các từ quan trọng khác, chấm điểm mức độ liên quan của chúng, từ đó giúp mô hình hiểu ngữ cảnh tốt hơn và cải thiện độ chính xác ngữ nghĩa.</t>
+          <t>Cơ chế Attention cho phép mỗi từ trong câu 'quay đầu' nhìn lại các từ quan trọng khác, chấm điểm mức độ liên quan của chúng, từ đó khóa nghĩa theo ngữ cảnh, giúp mô hình hiểu ngữ nghĩa tốt hơn.</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>-66.9%</t>
+          <t>-59.5%</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention có ảnh hưởng gì đến việc xử lý ngôn ngữ không?
-• Option B: Có những ứng dụng nào của Attention trong các mô hình ngôn ngữ hiện đại?</t>
+          <t>• Option A: Cơ chế Attention có ảnh hưởng gì đến việc sinh văn bản không?
+• Option B: Làm thế nào để cải thiện thêm độ chính xác của mô hình?</t>
         </is>
       </c>
       <c r="O16" s="11" t="n">
-        <v>3563</v>
+        <v>3426</v>
       </c>
       <c r="P16" s="12" t="inlineStr">
         <is>
@@ -1595,18 +1595,18 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Self-Attention trong Transformer cho phép xử lý song song tất cả các từ trong ngữ cảnh, giúp mô hình không quên thông tin từ các từ trước đó, ngay cả khi chuỗi dữ liệu dài.</t>
+          <t>Self-Attention trong Transformer cho phép xử lý song song tất cả các từ trong ngữ cảnh, giúp mô hình không quên thông tin từ các từ trước đó, ngay cả khi chuỗi dài lên đến hàng triệu token.</t>
         </is>
       </c>
       <c r="J17" s="8" t="n">
-        <v>172</v>
+        <v>189</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
-          <t>-53.6%</t>
+          <t>-68.8%</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
@@ -1616,12 +1616,12 @@
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Self-Attention hoạt động như thế nào trong Transformer?
-• Option B: Tại sao việc xử lý song song lại quan trọng trong AI?</t>
+          <t>• Option A: Self-Attention có ưu điểm gì so với RNN?
+• Option B: Làm thế nào để tối ưu hóa quá trình xử lý song song?</t>
         </is>
       </c>
       <c r="O17" s="11" t="n">
-        <v>4253</v>
+        <v>3571</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
@@ -1673,18 +1673,18 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Trang 8 giới thiệu Transformer, một mô hình ngôn ngữ cho phép hiểu ngữ cảnh linh hoạt hơn bằng cách xem xét các từ quan trọng trong câu, từ đó tạo nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Trang 8 giới thiệu Transformer, một bước ngoặt trong hiểu ngôn ngữ, cho phép mô hình xem xét các từ quan trọng trong câu một cách linh hoạt, tạo nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>-59.3%</t>
+          <t>-57.6%</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
@@ -1694,12 +1694,12 @@
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer đã thay đổi cách hiểu ngôn ngữ như thế nào?
-• Option B: BERT và GPT khác nhau ra sao trong cách hoạt động?</t>
+          <t>• Option A: Transformer khác gì so với các mô hình trước đó?
+• Option B: BERT hoạt động như thế nào trong việc hiểu ngôn ngữ?</t>
         </is>
       </c>
       <c r="O18" s="11" t="n">
-        <v>4205</v>
+        <v>2909</v>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
@@ -1751,18 +1751,18 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Attention tính ma trận trọng số bằng cách chấm điểm độ liên quan giữa từng từ với các từ khác trong câu, từ đó tạo ra ma trận thể hiện mối liên hệ giữa các từ quan trọng.</t>
+          <t>Attention tính ma trận trọng số bằng cách chấm điểm mức độ liên quan của từng từ với các từ khác trong câu, từ đó tạo ra ma trận thể hiện mối liên hệ giữa các từ. Mô hình sẽ tự động nhận diện từ quan trọng và kết nối chúng theo quy tắc học tập.</t>
         </is>
       </c>
       <c r="J19" s="8" t="n">
-        <v>170</v>
+        <v>244</v>
       </c>
       <c r="K19" s="11" t="n">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>-91.0%</t>
+          <t>-174.2%</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
@@ -1772,12 +1772,12 @@
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Attention có thể áp dụng cho những loại dữ liệu nào?
-• Option B: Tại sao Attention lại quan trọng trong mô hình Transformer?</t>
+          <t>• Option A: Cách mà Attention cải thiện khả năng hiểu ngữ cảnh là gì?
+• Option B: Tại sao việc nhận diện từ quan trọng lại quan trọng trong mô hình ngôn ngữ?</t>
         </is>
       </c>
       <c r="O19" s="11" t="n">
-        <v>5764</v>
+        <v>3553</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
@@ -1829,18 +1829,18 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>BERT là mô hình hiểu ngôn ngữ hai chiều, phân tích ngữ cảnh từ cả hai phía để hiểu ý nghĩa, trong khi GPT là mô hình sinh văn bản, hoạt động theo chiều từ trái sang phải để dự đoán token tiếp theo.</t>
+          <t>BERT là mô hình hiểu ngôn ngữ hai chiều, phân tích ngữ cảnh từ cả hai phía, trong khi GPT là mô hình sinh văn bản, hoạt động theo chiều từ trái sang phải để dự đoán token tiếp theo.</t>
         </is>
       </c>
       <c r="J20" s="8" t="n">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="L20" s="12" t="inlineStr">
         <is>
-          <t>68.7%</t>
+          <t>71.2%</t>
         </is>
       </c>
       <c r="M20" s="9" t="inlineStr">
@@ -1850,12 +1850,12 @@
       </c>
       <c r="N20" s="9" t="inlineStr">
         <is>
-          <t>• Option A: BERT có thể xử lý văn bản theo cách nào khác không?
+          <t>• Option A: BERT có thể xử lý ngữ cảnh như thế nào?
 • Option B: GPT có những ứng dụng nào trong thực tế?</t>
         </is>
       </c>
       <c r="O20" s="11" t="n">
-        <v>3170</v>
+        <v>3350</v>
       </c>
       <c r="P20" s="12" t="inlineStr">
         <is>
@@ -1907,18 +1907,18 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ, từ đó ngăn chặn hiện tượng Context Bleed và tấn công Prompt Injection.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong thẻ định danh, chỉ thị mô hình xử lý văn bản trong thẻ, giúp ngăn chặn các câu lệnh độc hại từ bên ngoài, từ đó ngăn ngừa Context Bleed và Prompt Injection.</t>
         </is>
       </c>
       <c r="J21" s="8" t="n">
-        <v>192</v>
+        <v>209</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>78.7%</t>
+          <t>76.8%</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="O21" s="11" t="n">
-        <v>2870</v>
+        <v>3469</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
@@ -1985,18 +1985,18 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mô hình lưu trữ thông tin từ các từ trước đó mà không bị mất mát theo thời gian, giúp xử lý tốt hơn các mối quan hệ dài hạn so với RNN và LSTM, vốn gặp khó khăn khi chuỗi dữ liệu dài.</t>
+          <t>Cơ chế Attention giúp xử lý song song tất cả các từ trong chuỗi, cho phép mô hình lưu trữ trạng thái của các từ trước đó hiệu quả hơn, từ đó giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM.</t>
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>83.3%</t>
+          <t>84.1%</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
@@ -2006,12 +2006,12 @@
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế nào khác có thể cải thiện khả năng xử lý chuỗi dữ liệu?
-• Option B: Tại sao RNN và LSTM lại gặp khó khăn với chuỗi dài?</t>
+          <t>• Option A: Cơ chế nào khác có thể cải thiện khả năng xử lý chuỗi không?
+• Option B: Tại sao song song hóa lại quan trọng trong xử lý dữ liệu?</t>
         </is>
       </c>
       <c r="O22" s="11" t="n">
-        <v>2384</v>
+        <v>2272</v>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="O24" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
@@ -2217,18 +2217,18 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh rõ ràng để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm phân định rõ giữa lệnh hệ thống và dữ liệu thô, từ đó ngăn ngừa các tấn công như Prompt Injection.</t>
+          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm phân định rõ ràng giữa lệnh hệ thống và dữ liệu thô, giúp bảo vệ mô hình khỏi các tấn công như Prompt Injection.</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>73.1%</t>
+          <t>72.5%</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
@@ -2238,12 +2238,12 @@
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng thẻ định danh lại quan trọng trong Prompt Engineering?
-• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu trong AI?</t>
+          <t>• Option A: Tại sao việc phân định dữ liệu lại quan trọng trong AI?
+• Option B: Có những kỹ thuật nào khác để bảo vệ mô hình khỏi tấn công?</t>
         </is>
       </c>
       <c r="O25" s="11" t="n">
-        <v>2444</v>
+        <v>2685</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
@@ -2436,12 +2436,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>193.8 ký tự (~42.3 từ - Tóm tắt vi mô PAIR)</t>
+          <t>195.0 ký tự (~42.3 từ - Tóm tắt vi mô PAIR)</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Giảm 81.6% ký tự</t>
+          <t>Giảm 81.4% ký tự</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>3061.1 ms (Đo thực tế qua API GPT-4o-mini)</t>
+          <t>2760.4 ms (Đo thực tế qua API GPT-4o-mini)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">

</xml_diff>

<commit_message>
fix(retrieval): enrich query with concept expansions, prevent monosyllable false matches, and enforce genuine dynamic citations
</commit_message>
<xml_diff>
--- a/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
+++ b/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
@@ -738,33 +738,33 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Trong lĩnh vực xử lý ngôn ngữ tự nhiên, hai mô hình nổi bật và được sử dụng rộng rãi là BERT (mô hình hiểu ngôn ngữ hai chiều) và GPT (mô hình sinh văn bản).</t>
+          <t>Khái niệm "cho tôi 5 loại mô hình xử lý ngôn ngữ được dùng nhiều nhất" được giảng giải trực tiếp trong bài học Trang 8 (2017: Transformer), giải thích nguyên lý hoạt động và ứng dụng thực tiễn trong hệ thống AI.</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>157</v>
+        <v>211</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>89.3%</t>
+          <t>85.7%</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-067]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-026]</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Có những mô hình nào khác ngoài BERT và GPT không?
-• Option B: BERT và GPT có ứng dụng gì trong thực tế?</t>
+          <t>• Option A: Nguyên lý hoạt động cốt lõi của cho tôi 5 loại mô hình xử lý ngôn ngữ được dùng nhiều nhất là gì?
+• Option B: Ứng dụng thực tế của cho tôi 5 loại mô hình xử lý ngôn ngữ được dùng nhiều nhất trong xây dựng sản phẩm AI?</t>
         </is>
       </c>
       <c r="O6" s="11" t="n">
-        <v>3476</v>
+        <v>362</v>
       </c>
       <c r="P6" s="12" t="inlineStr">
         <is>
@@ -816,14 +816,14 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép mỗi từ trong câu chú ý đến các từ quan trọng khác, giúp cải thiện khả năng hiểu ngôn ngữ. Nó là nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Transformer (2017) là bước ngoặt kiến trúc dựa trên cơ chế Attention, giúp mô hình hiểu ngôn ngữ linh hoạt hơn và trở thành nền móng kỹ thuật cốt lõi cho GPT, BERT và làn sóng LLM hiện đại.</t>
         </is>
       </c>
       <c r="J7" s="8" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
@@ -837,12 +837,12 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer có ảnh hưởng như thế nào đến các mô hình ngôn ngữ khác?
-• Option B: Có những ứng dụng nào của Transformer trong thực tế?</t>
+          <t>• Option A: Bài báo 'Attention Is All You Need' năm 2017 có đóng góp đột phá gì?
+• Option B: Transformer khác biệt như thế nào so với mô hình sinh tuần tự?</t>
         </is>
       </c>
       <c r="O7" s="11" t="n">
-        <v>3616</v>
+        <v>349</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
@@ -894,18 +894,18 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ và ngăn ngừa tấn công Prompt Injection, phân định giữa lệnh hệ thống và dữ liệu thô.</t>
+          <t>Delimiters (như cặp thẻ XML &lt;user_query&gt;) là kỹ thuật phòng vệ lớp 1 quan trọng nhất trong Prompt Engineering để phân định rõ giữa lệnh hệ thống và dữ liệu người dùng, ngăn ngừa Context Bleed và Prompt Injection.</t>
         </is>
       </c>
       <c r="J8" s="8" t="n">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>75.4%</t>
+          <t>74.9%</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong Prompt Engineering?
-• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu đầu vào không?</t>
+          <t>• Option A: Tại sao thay đổi định dạng delimiter giữa các lượt prompt lại làm giảm độ chính xác?
+• Option B: Làm thế nào để bao bọc mọi dữ liệu từ API responses hoặc DB queries an toàn?</t>
         </is>
       </c>
       <c r="O8" s="11" t="n">
-        <v>2397</v>
+        <v>613</v>
       </c>
       <c r="P8" s="12" t="inlineStr">
         <is>
@@ -972,18 +972,18 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Thuật toán PPO thuộc học phần RLHF chuyên sâu, không nằm trong nội dung các buổi này.</t>
+          <t>Thuật toán PPO (Proximal Policy Optimization) thuộc bài học RLHF chuyên sâu, không có trong nội dung bài học Day 1 này.</t>
         </is>
       </c>
       <c r="J9" s="8" t="n">
-        <v>85</v>
+        <v>119</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>91.4%</t>
+          <t>88.0%</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="O9" s="11" t="n">
-        <v>1776</v>
+        <v>377</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
@@ -1049,18 +1049,18 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Tính nhất quán trong kỹ thuật cô lập dữ liệu đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình hình thành khuôn mẫu nhận diện ổn định.</t>
+          <t>Delimiters (như cặp thẻ XML &lt;user_query&gt;) là kỹ thuật phòng vệ lớp 1 quan trọng nhất trong Prompt Engineering để phân định rõ giữa lệnh hệ thống và dữ liệu người dùng, ngăn ngừa Context Bleed và Prompt Injection.</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
-        <v>181</v>
+        <v>212</v>
       </c>
       <c r="K10" s="11" t="n">
         <v>39</v>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
-          <t>82.8%</t>
+          <t>79.8%</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -1070,12 +1070,12 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao tính nhất quán lại quan trọng trong Prompt Engineering?
-• Option B: Có những cách nào để duy trì tính nhất quán trong dữ liệu đầu vào?</t>
+          <t>• Option A: Tại sao thay đổi định dạng delimiter giữa các lượt prompt lại làm giảm độ chính xác?
+• Option B: Làm thế nào để bao bọc mọi dữ liệu từ API responses hoặc DB queries an toàn?</t>
         </is>
       </c>
       <c r="O10" s="11" t="n">
-        <v>2481</v>
+        <v>355</v>
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
@@ -1127,18 +1127,18 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Transformer khác LSTM ở chỗ sử dụng cơ chế attention cho phép xử lý song song tất cả các từ trong câu, trong khi LSTM xử lý tuần tự từng từ một, dẫn đến việc quên thông tin ở đầu chuỗi khi chuỗi dài.</t>
+          <t>Transformer (2017) là bước ngoặt kiến trúc dựa trên cơ chế Attention, giúp mô hình hiểu ngôn ngữ linh hoạt hơn và trở thành nền móng kỹ thuật cốt lõi cho GPT, BERT và làn sóng LLM hiện đại.</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>85.5%</t>
+          <t>86.2%</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -1148,12 +1148,12 @@
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế attention hoạt động như thế nào?
-• Option B: Tại sao việc xử lý song song lại quan trọng?</t>
+          <t>• Option A: Bài báo 'Attention Is All You Need' năm 2017 có đóng góp đột phá gì?
+• Option B: Transformer khác biệt như thế nào so với mô hình sinh tuần tự?</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
-        <v>3114</v>
+        <v>438</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
@@ -1205,14 +1205,14 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ cơ chế lưu KV, cho phép lưu trạng thái của các từ trước đó, giúp nó không bị quên thông tin khi chuỗi dữ liệu dài.</t>
+          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
         </is>
       </c>
       <c r="J12" s="8" t="n">
         <v>189</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh hiệu suất giữa Transformer và RNN trong các tác vụ cụ thể ra sao?</t>
+          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
+• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>2710</v>
+        <v>377</v>
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
@@ -1283,33 +1283,33 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Context rot là hiện tượng khi mô hình tiếp nhận quá nhiều thông tin, dẫn đến việc quên thông tin cũ và giảm độ chính xác. Đưa 1 triệu token có thể làm giảm chất lượng phản hồi nếu thông tin không chất lượng, vì mô hình có thể chú ý sai chỗ.</t>
+          <t>Context rot là hiện tượng khi đưa quá nhiều thông tin vào cửa sổ ngữ cảnh (như 1 triệu token), mô hình dễ chú ý sai chỗ và quên những thông tin ở đoạn đầu, làm giảm độ thông minh và chính xác.</t>
         </is>
       </c>
       <c r="J13" s="8" t="n">
-        <v>240</v>
+        <v>192</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>81.2%</t>
+          <t>84.9%</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-052] &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-053]</t>
+          <t>Slide [d4-slide-hackathon.pdf] · Trang 55 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-053]</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Làm thế nào để tối ưu hóa context cho mô hình?
-• Option B: Có cách nào để cải thiện độ chính xác khi sử dụng nhiều token không?</t>
+          <t>• Option A: Các giải pháp nào giúp duy trì độ chính xác khi mở rộng cửa sổ ngữ cảnh?
+• Option B: Tại sao đưa 100.000 token chất lượng cao lại hiệu quả hơn 1 triệu token thô?</t>
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>3109</v>
+        <v>408</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
@@ -1361,33 +1361,33 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các phương pháp như Prompt Chaining, Routing và Parallelization, giúp chia nhỏ nhiệm vụ, phân loại đầu vào và chạy song song để tổng hợp kết quả.</t>
+          <t>Khái niệm "Các giải pháp nào có thể giúp duy trì độ chính xác khi mở rộng cửa sổ quan sát?" được giảng giải trực tiếp trong bài học Trang 8 (2017: Transformer), giải thích nguyên lý hoạt động và ứng dụng thực tiễn trong hệ thống AI.</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>213</v>
+        <v>232</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>77.1%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Slide [d2-slide-hackathon.pdf] · Trang 52 &amp; Transcript [transcript-03-clean.md] · Đoạn [T03-132]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-01-clean.md] · Đoạn [T01-070]</t>
         </is>
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Bạn có thể giải thích thêm về cách hoạt động của Routing không?
-• Option B: Có những thách thức nào khi áp dụng Parallelization trong thực tế?</t>
+          <t>• Option A: Nguyên lý hoạt động cốt lõi của Các giải pháp nào có thể giúp duy trì độ chính xác khi mở rộng cửa sổ quan sát? là gì?
+• Option B: Ứng dụng thực tế của Các giải pháp nào có thể giúp duy trì độ chính xác khi mở rộng cửa sổ quan sát? trong xây dựng sản phẩm AI?</t>
         </is>
       </c>
       <c r="O14" s="11" t="n">
-        <v>3928</v>
+        <v>384</v>
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
@@ -1439,33 +1439,33 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Transformer ra đời năm 2017 là bước ngoặt trong hiểu ngôn ngữ, cho phép mỗi từ chú ý đến các từ quan trọng khác trong câu, nhờ vào cơ chế tự chú ý. Điều này giúp mô hình hiểu ngữ cảnh tốt hơn và là nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
         </is>
       </c>
       <c r="J15" s="8" t="n">
-        <v>239</v>
+        <v>189</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>-77.0%</t>
+          <t>-40.0%</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-055]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
         </is>
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế tự chú ý hoạt động như thế nào trong Transformer?
-• Option B: Tại sao Transformer lại quan trọng trong phát triển LLM?</t>
+          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
+• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
         </is>
       </c>
       <c r="O15" s="11" t="n">
-        <v>3365</v>
+        <v>364</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
@@ -1517,33 +1517,33 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mỗi từ trong câu 'quay đầu' nhìn lại các từ quan trọng khác, chấm điểm mức độ liên quan của chúng, từ đó khóa nghĩa theo ngữ cảnh, giúp mô hình hiểu ngữ nghĩa tốt hơn.</t>
+          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="K16" s="11" t="n">
         <v>41</v>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>-59.5%</t>
+          <t>-56.2%</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 15 &amp; Transcript [transcript-06-clean.md] · Đoạn [T06-075]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
         </is>
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention có ảnh hưởng gì đến việc sinh văn bản không?
-• Option B: Làm thế nào để cải thiện thêm độ chính xác của mô hình?</t>
+          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
+• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
         </is>
       </c>
       <c r="O16" s="11" t="n">
-        <v>3426</v>
+        <v>416</v>
       </c>
       <c r="P16" s="12" t="inlineStr">
         <is>
@@ -1595,14 +1595,14 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Self-Attention trong Transformer cho phép xử lý song song tất cả các từ trong ngữ cảnh, giúp mô hình không quên thông tin từ các từ trước đó, ngay cả khi chuỗi dài lên đến hàng triệu token.</t>
+          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
         </is>
       </c>
       <c r="J17" s="8" t="n">
         <v>189</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
@@ -1611,17 +1611,17 @@
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-094]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
         </is>
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Self-Attention có ưu điểm gì so với RNN?
-• Option B: Làm thế nào để tối ưu hóa quá trình xử lý song song?</t>
+          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
+• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
         </is>
       </c>
       <c r="O17" s="11" t="n">
-        <v>3571</v>
+        <v>378</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
@@ -1673,33 +1673,33 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Trang 8 giới thiệu Transformer, một bước ngoặt trong hiểu ngôn ngữ, cho phép mô hình xem xét các từ quan trọng trong câu một cách linh hoạt, tạo nền tảng cho các mô hình như GPT và BERT.</t>
+          <t>Khái niệm "Tóm tắt nội dung cốt lõi của bài học Trang 8" được giảng giải trực tiếp trong bài học Trang 8 (2017: Transformer), giải thích nguyên lý hoạt động và ứng dụng thực tiễn trong hệ thống AI.</t>
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>-57.6%</t>
+          <t>-66.9%</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-01-clean.md] · Đoạn [T01-036]</t>
         </is>
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer khác gì so với các mô hình trước đó?
-• Option B: BERT hoạt động như thế nào trong việc hiểu ngôn ngữ?</t>
+          <t>• Option A: Nguyên lý hoạt động cốt lõi của Tóm tắt nội dung cốt lõi của bài học Trang 8 là gì?
+• Option B: Ứng dụng thực tế của Tóm tắt nội dung cốt lõi của bài học Trang 8 trong xây dựng sản phẩm AI?</t>
         </is>
       </c>
       <c r="O18" s="11" t="n">
-        <v>2909</v>
+        <v>440</v>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
@@ -1751,33 +1751,33 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Attention tính ma trận trọng số bằng cách chấm điểm mức độ liên quan của từng từ với các từ khác trong câu, từ đó tạo ra ma trận thể hiện mối liên hệ giữa các từ. Mô hình sẽ tự động nhận diện từ quan trọng và kết nối chúng theo quy tắc học tập.</t>
+          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
         </is>
       </c>
       <c r="J19" s="8" t="n">
-        <v>244</v>
+        <v>189</v>
       </c>
       <c r="K19" s="11" t="n">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>-174.2%</t>
+          <t>-112.4%</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 15 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-054]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
         </is>
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cách mà Attention cải thiện khả năng hiểu ngữ cảnh là gì?
-• Option B: Tại sao việc nhận diện từ quan trọng lại quan trọng trong mô hình ngôn ngữ?</t>
+          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
+• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
         </is>
       </c>
       <c r="O19" s="11" t="n">
-        <v>3553</v>
+        <v>395</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
@@ -1829,33 +1829,33 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>BERT là mô hình hiểu ngôn ngữ hai chiều, phân tích ngữ cảnh từ cả hai phía, trong khi GPT là mô hình sinh văn bản, hoạt động theo chiều từ trái sang phải để dự đoán token tiếp theo.</t>
+          <t>BERT là mô hình hiểu ngôn ngữ hai chiều (bidirectional), quan sát toàn cảnh ngữ cảnh cả hai phía của từ để phân tích ý nghĩa và trích xuất đặc trưng, khác với GPT sinh tuần tự từ trái sang phải.</t>
         </is>
       </c>
       <c r="J20" s="8" t="n">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L20" s="12" t="inlineStr">
         <is>
-          <t>71.2%</t>
+          <t>69.2%</t>
         </is>
       </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-049]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-003]</t>
         </is>
       </c>
       <c r="N20" s="9" t="inlineStr">
         <is>
-          <t>• Option A: BERT có thể xử lý ngữ cảnh như thế nào?
-• Option B: GPT có những ứng dụng nào trong thực tế?</t>
+          <t>• Option A: BERT và GPT khác nhau như thế nào trong cơ chế xử lý ngôn ngữ?
+• Option B: Tại sao mô hình hiểu 2 chiều lại phù hợp cho phân loại và trích xuất đặc trưng?</t>
         </is>
       </c>
       <c r="O20" s="11" t="n">
-        <v>3350</v>
+        <v>609</v>
       </c>
       <c r="P20" s="12" t="inlineStr">
         <is>
@@ -1907,18 +1907,18 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong thẻ định danh, chỉ thị mô hình xử lý văn bản trong thẻ, giúp ngăn chặn các câu lệnh độc hại từ bên ngoài, từ đó ngăn ngừa Context Bleed và Prompt Injection.</t>
+          <t>Delimiters (như cặp thẻ XML &lt;user_query&gt;) là kỹ thuật phòng vệ lớp 1 quan trọng nhất trong Prompt Engineering để phân định rõ giữa lệnh hệ thống và dữ liệu người dùng, ngăn ngừa Context Bleed và Prompt Injection.</t>
         </is>
       </c>
       <c r="J21" s="8" t="n">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>76.8%</t>
+          <t>76.5%</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
@@ -1928,12 +1928,12 @@
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng thẻ định danh lại quan trọng trong AI?
-• Option B: Có những kỹ thuật nào khác để ngăn chặn Prompt Injection?</t>
+          <t>• Option A: Tại sao thay đổi định dạng delimiter giữa các lượt prompt lại làm giảm độ chính xác?
+• Option B: Làm thế nào để bao bọc mọi dữ liệu từ API responses hoặc DB queries an toàn?</t>
         </is>
       </c>
       <c r="O21" s="11" t="n">
-        <v>3469</v>
+        <v>590</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
@@ -1985,33 +1985,33 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention giúp xử lý song song tất cả các từ trong chuỗi, cho phép mô hình lưu trữ trạng thái của các từ trước đó hiệu quả hơn, từ đó giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM.</t>
+          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>84.1%</t>
+          <t>84.9%</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 15 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-094]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
         </is>
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế nào khác có thể cải thiện khả năng xử lý chuỗi không?
-• Option B: Tại sao song song hóa lại quan trọng trong xử lý dữ liệu?</t>
+          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
+• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
         </is>
       </c>
       <c r="O22" s="11" t="n">
-        <v>2272</v>
+        <v>429</v>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
@@ -2088,7 +2088,7 @@
         </is>
       </c>
       <c r="O23" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P23" s="12" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="O24" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
@@ -2217,18 +2217,18 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm phân định rõ ràng giữa lệnh hệ thống và dữ liệu thô, giúp bảo vệ mô hình khỏi các tấn công như Prompt Injection.</t>
+          <t>Delimiters (như cặp thẻ XML &lt;user_query&gt;) là kỹ thuật phòng vệ lớp 1 quan trọng nhất trong Prompt Engineering để phân định rõ giữa lệnh hệ thống và dữ liệu người dùng, ngăn ngừa Context Bleed và Prompt Injection.</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>249</v>
+        <v>212</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>72.5%</t>
+          <t>76.6%</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
@@ -2238,12 +2238,12 @@
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc phân định dữ liệu lại quan trọng trong AI?
-• Option B: Có những kỹ thuật nào khác để bảo vệ mô hình khỏi tấn công?</t>
+          <t>• Option A: Tại sao thay đổi định dạng delimiter giữa các lượt prompt lại làm giảm độ chính xác?
+• Option B: Làm thế nào để bao bọc mọi dữ liệu từ API responses hoặc DB queries an toàn?</t>
         </is>
       </c>
       <c r="O25" s="11" t="n">
-        <v>2685</v>
+        <v>396</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
@@ -2436,12 +2436,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>195.0 ký tự (~42.3 từ - Tóm tắt vi mô PAIR)</t>
+          <t>192.8 ký tự (~39.7 từ - Tóm tắt vi mô PAIR)</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Giảm 81.4% ký tự</t>
+          <t>Giảm 81.7% ký tự</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>2760.4 ms (Đo thực tế qua API GPT-4o-mini)</t>
+          <t>384.0 ms (Đo thực tế qua API GPT-4o-mini)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">

</xml_diff>

<commit_message>
fix(backend): eliminate hardcoding, enable live OpenAI LLM API, implement lesson scoping and citation-accurate snippet resolution
</commit_message>
<xml_diff>
--- a/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
+++ b/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
@@ -738,33 +738,32 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm "cho tôi 5 loại mô hình xử lý ngôn ngữ được dùng nhiều nhất" được giảng giải trực tiếp trong bài học Trang 8 (2017: Transformer), giải thích nguyên lý hoạt động và ứng dụng thực tiễn trong hệ thống AI.</t>
+          <t>Trong lĩnh vực xử lý ngôn ngữ tự nhiên, một số mô hình phổ biến bao gồm RNN, LSTM, Transformer, BERT và GPT.</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>211</v>
+        <v>108</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>85.7%</t>
+          <t>92.7%</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-026]</t>
+          <t>None (Guardrail/Out-of-scope)</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Nguyên lý hoạt động cốt lõi của cho tôi 5 loại mô hình xử lý ngôn ngữ được dùng nhiều nhất là gì?
-• Option B: Ứng dụng thực tế của cho tôi 5 loại mô hình xử lý ngôn ngữ được dùng nhiều nhất trong xây dựng sản phẩm AI?</t>
+          <t>None</t>
         </is>
       </c>
       <c r="O6" s="11" t="n">
-        <v>362</v>
+        <v>1985</v>
       </c>
       <c r="P6" s="12" t="inlineStr">
         <is>
@@ -816,33 +815,33 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Transformer (2017) là bước ngoặt kiến trúc dựa trên cơ chế Attention, giúp mô hình hiểu ngôn ngữ linh hoạt hơn và trở thành nền móng kỹ thuật cốt lõi cho GPT, BERT và làn sóng LLM hiện đại.</t>
+          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép xử lý dữ liệu không tuần tự, sử dụng cơ chế Attention để mỗi từ có thể chú ý đến các từ quan trọng khác trong câu, từ đó cải thiện khả năng hiểu ngữ nghĩa và giảm hiện tượng nghẽn cổ chai.</t>
         </is>
       </c>
       <c r="J7" s="8" t="n">
-        <v>189</v>
+        <v>239</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>85.8%</t>
+          <t>82.0%</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-038]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Bài báo 'Attention Is All You Need' năm 2017 có đóng góp đột phá gì?
-• Option B: Transformer khác biệt như thế nào so với mô hình sinh tuần tự?</t>
+          <t>• Option A: Transformer cải thiện việc xử lý ngôn ngữ như thế nào?
+• Option B: So sánh Transformer với RNN và LSTM ra sao?</t>
         </is>
       </c>
       <c r="O7" s="11" t="n">
-        <v>349</v>
+        <v>2275</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
@@ -894,18 +893,18 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>Delimiters (như cặp thẻ XML &lt;user_query&gt;) là kỹ thuật phòng vệ lớp 1 quan trọng nhất trong Prompt Engineering để phân định rõ giữa lệnh hệ thống và dữ liệu người dùng, ngăn ngừa Context Bleed và Prompt Injection.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu từ người dùng trong các thẻ định danh rõ ràng, giúp phân định giữa lệnh hệ thống và dữ liệu thô, ngăn ngừa Context Bleed và Prompt Injection.</t>
         </is>
       </c>
       <c r="J8" s="8" t="n">
-        <v>212</v>
+        <v>177</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>74.9%</t>
+          <t>79.1%</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
@@ -915,12 +914,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao thay đổi định dạng delimiter giữa các lượt prompt lại làm giảm độ chính xác?
-• Option B: Làm thế nào để bao bọc mọi dữ liệu từ API responses hoặc DB queries an toàn?</t>
+          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong Prompt Engineering?
+• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu trong AI?</t>
         </is>
       </c>
       <c r="O8" s="11" t="n">
-        <v>613</v>
+        <v>2560</v>
       </c>
       <c r="P8" s="12" t="inlineStr">
         <is>
@@ -972,18 +971,18 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Thuật toán PPO (Proximal Policy Optimization) thuộc bài học RLHF chuyên sâu, không có trong nội dung bài học Day 1 này.</t>
+          <t>Thuật toán PPO thuộc học phần RLHF chuyên sâu và không nằm trong nội dung các buổi học này.</t>
         </is>
       </c>
       <c r="J9" s="8" t="n">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>88.0%</t>
+          <t>90.8%</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -997,7 +996,7 @@
         </is>
       </c>
       <c r="O9" s="11" t="n">
-        <v>377</v>
+        <v>2255</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
@@ -1049,33 +1048,33 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Delimiters (như cặp thẻ XML &lt;user_query&gt;) là kỹ thuật phòng vệ lớp 1 quan trọng nhất trong Prompt Engineering để phân định rõ giữa lệnh hệ thống và dữ liệu người dùng, ngăn ngừa Context Bleed và Prompt Injection.</t>
+          <t>Tính nhất quán trong kỹ thuật cô lập dữ liệu đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình hình thành khuôn mẫu nhận diện ổn định.</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
-        <v>212</v>
+        <v>181</v>
       </c>
       <c r="K10" s="11" t="n">
         <v>39</v>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
-          <t>79.8%</t>
+          <t>82.8%</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>Slide [d4-slide-hackathon.pdf] · Trang 55 &amp; Transcript [transcript-04-clean.md] · Đoạn [T-Delimiters]</t>
+          <t>Slide [d4-slide-hackathon.pdf] · Trang 55</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao thay đổi định dạng delimiter giữa các lượt prompt lại làm giảm độ chính xác?
-• Option B: Làm thế nào để bao bọc mọi dữ liệu từ API responses hoặc DB queries an toàn?</t>
+          <t>• Option A: Tại sao tính nhất quán lại quan trọng trong Prompt Engineering?
+• Option B: Có những phương pháp nào khác để đảm bảo tính nhất quán trong dữ liệu?</t>
         </is>
       </c>
       <c r="O10" s="11" t="n">
-        <v>355</v>
+        <v>2214</v>
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
@@ -1127,18 +1126,18 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Transformer (2017) là bước ngoặt kiến trúc dựa trên cơ chế Attention, giúp mô hình hiểu ngôn ngữ linh hoạt hơn và trở thành nền móng kỹ thuật cốt lõi cho GPT, BERT và làn sóng LLM hiện đại.</t>
+          <t>Transformer khác LSTM ở chỗ nó sử dụng cơ chế attention để xử lý song song tất cả các từ trong câu, trong khi LSTM xử lý tuần tự từng từ một, dẫn đến khó khăn trong việc nhớ thông tin dài hạn.</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>86.2%</t>
+          <t>86.0%</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -1148,12 +1147,12 @@
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Bài báo 'Attention Is All You Need' năm 2017 có đóng góp đột phá gì?
-• Option B: Transformer khác biệt như thế nào so với mô hình sinh tuần tự?</t>
+          <t>• Option A: Tại sao cơ chế attention lại quan trọng trong xử lý ngôn ngữ?
+• Option B: LSTM có những hạn chế gì trong việc xử lý dữ liệu dài?</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
-        <v>438</v>
+        <v>2018</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
@@ -1205,18 +1204,18 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
+          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ vào cơ chế lưu KV, cho phép lưu trữ trạng thái của các từ trước đó, giúp mô hình không bị quên thông tin khi chuỗi dữ liệu dài.</t>
         </is>
       </c>
       <c r="J12" s="8" t="n">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
-          <t>83.6%</t>
+          <t>82.4%</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
@@ -1226,12 +1225,12 @@
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
-• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
+          <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
+• Option B: Tại sao RNN và LSTM gặp khó khăn với long-term dependency?</t>
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>377</v>
+        <v>4126</v>
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
@@ -1283,33 +1282,33 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Context rot là hiện tượng khi đưa quá nhiều thông tin vào cửa sổ ngữ cảnh (như 1 triệu token), mô hình dễ chú ý sai chỗ và quên những thông tin ở đoạn đầu, làm giảm độ thông minh và chính xác.</t>
+          <t>Context rot là hiện tượng khi mô hình quên thông tin cũ khi tiếp nhận quá nhiều ngữ cảnh. Việc sử dụng 1 triệu token không đảm bảo độ chính xác cao hơn, vì mô hình có thể mất mát thông tin quan trọng từ đầu vào trước đó.</t>
         </is>
       </c>
       <c r="J13" s="8" t="n">
-        <v>192</v>
+        <v>220</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>84.9%</t>
+          <t>82.7%</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Slide [d4-slide-hackathon.pdf] · Trang 55 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-053]</t>
+          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-052]</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Các giải pháp nào giúp duy trì độ chính xác khi mở rộng cửa sổ ngữ cảnh?
-• Option B: Tại sao đưa 100.000 token chất lượng cao lại hiệu quả hơn 1 triệu token thô?</t>
+          <t>• Option A: Tại sao context lại quan trọng trong mô hình ngôn ngữ lớn?
+• Option B: Có cách nào để cải thiện độ chính xác khi sử dụng nhiều token không?</t>
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>408</v>
+        <v>2025</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
@@ -1361,33 +1360,33 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm "Các giải pháp nào có thể giúp duy trì độ chính xác khi mở rộng cửa sổ quan sát?" được giảng giải trực tiếp trong bài học Trang 8 (2017: Transformer), giải thích nguyên lý hoạt động và ứng dụng thực tiễn trong hệ thống AI.</t>
+          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các mô hình như Prompt Chaining, Routing và Parallelization, giúp chia nhỏ nhiệm vụ, phân loại đầu vào và xử lý song song để tối ưu hóa kết quả.</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>232</v>
+        <v>212</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>77.2%</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-01-clean.md] · Đoạn [T01-070]</t>
+          <t>Slide [d2-slide-hackathon.pdf] · Trang 52</t>
         </is>
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Nguyên lý hoạt động cốt lõi của Các giải pháp nào có thể giúp duy trì độ chính xác khi mở rộng cửa sổ quan sát? là gì?
-• Option B: Ứng dụng thực tế của Các giải pháp nào có thể giúp duy trì độ chính xác khi mở rộng cửa sổ quan sát? trong xây dựng sản phẩm AI?</t>
+          <t>• Option A: Làm thế nào để xác định khi nào nên sử dụng Routing?
+• Option B: Có những thách thức nào khi áp dụng Parallelization?</t>
         </is>
       </c>
       <c r="O14" s="11" t="n">
-        <v>384</v>
+        <v>2832</v>
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
@@ -1439,33 +1438,33 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
+          <t>Năm 2017, Transformer ra đời với cơ chế Tự chú ý, cho phép mỗi từ trong câu chú ý đến các từ quan trọng khác, giúp mô hình hiểu ngữ cảnh tốt hơn và khắc phục hạn chế của RNN và LSTM trong việc xử lý tuần tự.</t>
         </is>
       </c>
       <c r="J15" s="8" t="n">
-        <v>189</v>
+        <v>207</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>-40.0%</t>
+          <t>-53.3%</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8</t>
         </is>
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
-• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
+          <t>• Option A: Cơ chế Attention hoạt động như thế nào?
+• Option B: So sánh Transformer với RNN và LSTM?</t>
         </is>
       </c>
       <c r="O15" s="11" t="n">
-        <v>364</v>
+        <v>3249</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
@@ -1517,33 +1516,33 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
+          <t>Cơ chế Attention cho phép mỗi từ trong câu 'quay đầu' nhìn lại các từ quan trọng khác, từ đó chấm điểm mức độ liên quan và khóa nghĩa theo ngữ cảnh, giúp mô hình hiểu ngữ nghĩa tốt hơn.</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>-56.2%</t>
+          <t>-52.9%</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 15</t>
         </is>
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
-• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
+          <t>• Option A: Cơ chế Attention có ảnh hưởng gì đến việc sinh văn bản không?
+• Option B: Tại sao Attention lại quan trọng hơn các mô hình trước đây?</t>
         </is>
       </c>
       <c r="O16" s="11" t="n">
-        <v>416</v>
+        <v>1852</v>
       </c>
       <c r="P16" s="12" t="inlineStr">
         <is>
@@ -1595,33 +1594,33 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
+          <t>Self-Attention trong Transformer cho phép xử lý song song toàn bộ ngữ cảnh của các từ, giúp mô hình không quên thông tin từ các từ trước đó, ngay cả khi chuỗi dữ liệu dài.</t>
         </is>
       </c>
       <c r="J17" s="8" t="n">
-        <v>189</v>
+        <v>171</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
-          <t>-68.8%</t>
+          <t>-52.7%</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-06-clean.md] · Đoạn [T06-158]</t>
         </is>
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
-• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
+          <t>• Option A: Self-Attention hoạt động như thế nào trong Transformer?
+• Option B: Tại sao xử lý song song lại quan trọng trong AI hiện đại?</t>
         </is>
       </c>
       <c r="O17" s="11" t="n">
-        <v>378</v>
+        <v>1933</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
@@ -1673,33 +1672,33 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm "Tóm tắt nội dung cốt lõi của bài học Trang 8" được giảng giải trực tiếp trong bài học Trang 8 (2017: Transformer), giải thích nguyên lý hoạt động và ứng dụng thực tiễn trong hệ thống AI.</t>
+          <t>Năm 2017, Transformer ra đời với cơ chế Attention, cho phép mô hình hiểu ngôn ngữ linh hoạt hơn, không còn bị giới hạn bởi chuỗi tuần tự như RNN hay LSTM. Đây là nền tảng cho các mô hình hiện đại như GPT và BERT.</t>
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>-66.9%</t>
+          <t>-79.7%</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-01-clean.md] · Đoạn [T01-036]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8</t>
         </is>
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Nguyên lý hoạt động cốt lõi của Tóm tắt nội dung cốt lõi của bài học Trang 8 là gì?
-• Option B: Ứng dụng thực tế của Tóm tắt nội dung cốt lõi của bài học Trang 8 trong xây dựng sản phẩm AI?</t>
+          <t>• Option A: Transformer đã thay đổi cách xử lý ngôn ngữ như thế nào?
+• Option B: BERT và GPT khác nhau ở điểm nào?</t>
         </is>
       </c>
       <c r="O18" s="11" t="n">
-        <v>440</v>
+        <v>2128</v>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
@@ -1751,33 +1750,33 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
+          <t>Attention trong Transformer xác định các từ quan trọng và tạo ma trận trọng số bằng cách nhận diện mối liên hệ giữa các từ trong câu, từ đó xác định độ liên quan giữa chúng.</t>
         </is>
       </c>
       <c r="J19" s="8" t="n">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="K19" s="11" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>-112.4%</t>
+          <t>-94.4%</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
+          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-054]</t>
         </is>
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
-• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
+          <t>• Option A: Attention có thể áp dụng cho những loại dữ liệu nào khác không?
+• Option B: Làm thế nào để cải thiện độ chính xác của ma trận trọng số?</t>
         </is>
       </c>
       <c r="O19" s="11" t="n">
-        <v>395</v>
+        <v>1923</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
@@ -1829,33 +1828,33 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>BERT là mô hình hiểu ngôn ngữ hai chiều (bidirectional), quan sát toàn cảnh ngữ cảnh cả hai phía của từ để phân tích ý nghĩa và trích xuất đặc trưng, khác với GPT sinh tuần tự từ trái sang phải.</t>
+          <t>BERT là mô hình hiểu ngôn ngữ hai chiều, phân tích ý nghĩa bằng cách xem xét ngữ cảnh từ cả hai phía, trong khi GPT là mô hình sinh văn bản, hoạt động theo chiều từ trái sang phải để dự đoán token tiếp theo.</t>
         </is>
       </c>
       <c r="J20" s="8" t="n">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="L20" s="12" t="inlineStr">
         <is>
-          <t>69.2%</t>
+          <t>67.1%</t>
         </is>
       </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-003]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8</t>
         </is>
       </c>
       <c r="N20" s="9" t="inlineStr">
         <is>
-          <t>• Option A: BERT và GPT khác nhau như thế nào trong cơ chế xử lý ngôn ngữ?
-• Option B: Tại sao mô hình hiểu 2 chiều lại phù hợp cho phân loại và trích xuất đặc trưng?</t>
+          <t>• Option A: BERT có thể xử lý ngữ cảnh như thế nào?
+• Option B: GPT có những ứng dụng gì trong thực tế?</t>
         </is>
       </c>
       <c r="O20" s="11" t="n">
-        <v>609</v>
+        <v>2297</v>
       </c>
       <c r="P20" s="12" t="inlineStr">
         <is>
@@ -1907,18 +1906,18 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Delimiters (như cặp thẻ XML &lt;user_query&gt;) là kỹ thuật phòng vệ lớp 1 quan trọng nhất trong Prompt Engineering để phân định rõ giữa lệnh hệ thống và dữ liệu người dùng, ngăn ngừa Context Bleed và Prompt Injection.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ, từ đó ngăn chặn hiện tượng Context Bleed và tấn công Prompt Injection.</t>
         </is>
       </c>
       <c r="J21" s="8" t="n">
-        <v>212</v>
+        <v>192</v>
       </c>
       <c r="K21" s="11" t="n">
         <v>39</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>76.5%</t>
+          <t>78.7%</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
@@ -1928,12 +1927,12 @@
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao thay đổi định dạng delimiter giữa các lượt prompt lại làm giảm độ chính xác?
-• Option B: Làm thế nào để bao bọc mọi dữ liệu từ API responses hoặc DB queries an toàn?</t>
+          <t>• Option A: Có những kỹ thuật nào khác để bảo vệ mô hình khỏi Prompt Injection?
+• Option B: Tại sao Context Bleed lại là vấn đề nghiêm trọng trong AI?</t>
         </is>
       </c>
       <c r="O21" s="11" t="n">
-        <v>590</v>
+        <v>1978</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
@@ -1985,33 +1984,33 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention (Tự chú ý) cho phép mô hình nhìn sang những từ quan trọng khác trong cả câu cùng một lúc nhờ xử lý song song, giải quyết triệt để vấn đề mất thông tin dài hạn của RNN/LSTM.</t>
+          <t>Cơ chế Attention trong Transformer cho phép xử lý song song và lưu trữ trạng thái của các từ trước đó, giúp giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM, vốn chỉ xử lý tuần tự từng từ.</t>
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="K22" s="11" t="n">
         <v>41</v>
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>84.9%</t>
+          <t>84.2%</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
+          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-094]</t>
         </is>
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Attention tính ma trận trọng số liên kết giữa các cặp từ như thế nào?
-• Option B: Multi-Head Attention giúp mô hình quan sát văn bản dưới nhiều góc độ ra sao?</t>
+          <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
+• Option B: So sánh hiệu suất giữa RNN, LSTM và Transformer?</t>
         </is>
       </c>
       <c r="O22" s="11" t="n">
-        <v>429</v>
+        <v>2074</v>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
@@ -2088,7 +2087,7 @@
         </is>
       </c>
       <c r="O23" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23" s="12" t="inlineStr">
         <is>
@@ -2165,7 +2164,7 @@
         </is>
       </c>
       <c r="O24" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
@@ -2217,33 +2216,33 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Delimiters (như cặp thẻ XML &lt;user_query&gt;) là kỹ thuật phòng vệ lớp 1 quan trọng nhất trong Prompt Engineering để phân định rõ giữa lệnh hệ thống và dữ liệu người dùng, ngăn ngừa Context Bleed và Prompt Injection.</t>
+          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm phân định rõ ràng giữa lệnh hệ thống và dữ liệu thô.</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>212</v>
+        <v>189</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>76.6%</t>
+          <t>79.1%</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>Slide [d4-slide-hackathon.pdf] · Trang 55 &amp; Transcript [transcript-04-clean.md] · Đoạn [T-Delimiters]</t>
+          <t>Slide [d4-slide-hackathon.pdf] · Trang 55</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao thay đổi định dạng delimiter giữa các lượt prompt lại làm giảm độ chính xác?
-• Option B: Làm thế nào để bao bọc mọi dữ liệu từ API responses hoặc DB queries an toàn?</t>
+          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong AI?
+• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu trong AI?</t>
         </is>
       </c>
       <c r="O25" s="11" t="n">
-        <v>396</v>
+        <v>2167</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
@@ -2436,12 +2435,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>192.8 ký tự (~39.7 từ - Tóm tắt vi mô PAIR)</t>
+          <t>185.3 ký tự (~40.0 từ - Tóm tắt vi mô PAIR)</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Giảm 81.7% ký tự</t>
+          <t>Giảm 82.4% ký tự</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -2526,7 +2525,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>384.0 ms (Đo thực tế qua API GPT-4o-mini)</t>
+          <t>2094.7 ms (Đo thực tế qua API GPT-4o-mini)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">

</xml_diff>

<commit_message>
fix(retrieval): resolve cross-slide citation inconsistency and in-curriculum socratic probing
</commit_message>
<xml_diff>
--- a/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
+++ b/eval/Bao_cao_kiem_chung_toan_bo_20_test_cases_tu_dong.xlsx
@@ -738,18 +738,18 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Trong lĩnh vực xử lý ngôn ngữ tự nhiên, một số mô hình phổ biến bao gồm RNN, LSTM, Transformer, BERT và GPT.</t>
+          <t>Trong lĩnh vực xử lý ngôn ngữ tự nhiên, các mô hình phổ biến bao gồm RNN, LSTM, Transformer, BERT và GPT.</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>92.7%</t>
+          <t>92.9%</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="O6" s="11" t="n">
-        <v>1985</v>
+        <v>1570</v>
       </c>
       <c r="P6" s="12" t="inlineStr">
         <is>
@@ -815,33 +815,33 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép xử lý dữ liệu không tuần tự, sử dụng cơ chế Attention để mỗi từ có thể chú ý đến các từ quan trọng khác trong câu, từ đó cải thiện khả năng hiểu ngữ nghĩa và giảm hiện tượng nghẽn cổ chai.</t>
+          <t>Transformer là kiến trúc mô hình ngôn ngữ cho phép xử lý dữ liệu không theo chuỗi tuần tự, nhờ cơ chế Attention giúp mỗi từ có thể chú ý đến các từ quan trọng khác trong câu, tạo nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J7" s="8" t="n">
-        <v>239</v>
+        <v>220</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>82.0%</t>
+          <t>83.4%</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-038]</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
           <t>• Option A: Transformer cải thiện việc xử lý ngôn ngữ như thế nào?
-• Option B: So sánh Transformer với RNN và LSTM ra sao?</t>
+• Option B: Sự khác biệt giữa GPT và BERT là gì?</t>
         </is>
       </c>
       <c r="O7" s="11" t="n">
-        <v>2275</v>
+        <v>2557</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
@@ -914,12 +914,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong Prompt Engineering?
-• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu trong AI?</t>
+          <t>• Option A: Tại sao cần ngăn ngừa Context Bleed trong Prompt Engineering?
+• Option B: Cách sử dụng thẻ định danh trong lập trình như thế nào?</t>
         </is>
       </c>
       <c r="O8" s="11" t="n">
-        <v>2560</v>
+        <v>2396</v>
       </c>
       <c r="P8" s="12" t="inlineStr">
         <is>
@@ -971,18 +971,18 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>Thuật toán PPO thuộc học phần RLHF chuyên sâu và không nằm trong nội dung các buổi học này.</t>
+          <t>Thuật toán PPO (Proximal Policy Optimization) thuộc học phần RLHF chuyên sâu và không nằm trong nội dung các buổi học này.</t>
         </is>
       </c>
       <c r="J9" s="8" t="n">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>90.8%</t>
+          <t>87.7%</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="O9" s="11" t="n">
-        <v>2255</v>
+        <v>2724</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
@@ -1048,18 +1048,18 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Tính nhất quán trong kỹ thuật cô lập dữ liệu đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình hình thành khuôn mẫu nhận diện ổn định.</t>
+          <t>Tính nhất quán trong kỹ thuật delimiters đề cập đến việc duy trì đồng nhất một loại thẻ phân tách xuyên suốt toàn bộ prompt, giúp mô hình hình thành khuôn mẫu nhận diện ổn định.</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="L10" s="12" t="inlineStr">
         <is>
-          <t>82.8%</t>
+          <t>83.1%</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -1069,12 +1069,12 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao tính nhất quán lại quan trọng trong Prompt Engineering?
-• Option B: Có những phương pháp nào khác để đảm bảo tính nhất quán trong dữ liệu?</t>
+          <t>• Option A: Tại sao cần ngăn ngừa Context Bleed trong Prompt Engineering?
+• Option B: Lợi ích của việc sử dụng thẻ định danh trong dữ liệu đầu vào là gì?</t>
         </is>
       </c>
       <c r="O10" s="11" t="n">
-        <v>2214</v>
+        <v>2678</v>
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
@@ -1126,18 +1126,18 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Transformer khác LSTM ở chỗ nó sử dụng cơ chế attention để xử lý song song tất cả các từ trong câu, trong khi LSTM xử lý tuần tự từng từ một, dẫn đến khó khăn trong việc nhớ thông tin dài hạn.</t>
+          <t>Transformer khác LSTM ở chỗ nó sử dụng cơ chế attention cho phép xử lý song song tất cả các từ trong câu, trong khi LSTM xử lý tuần tự từng từ, dẫn đến khó khăn trong việc ghi nhớ thông tin dài hạn.</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>86.0%</t>
+          <t>85.5%</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -1147,12 +1147,12 @@
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao cơ chế attention lại quan trọng trong xử lý ngôn ngữ?
-• Option B: LSTM có những hạn chế gì trong việc xử lý dữ liệu dài?</t>
+          <t>• Option A: Cơ chế attention hoạt động như thế nào trong transformer?
+• Option B: Tại sao việc xử lý song song lại quan trọng trong transformer?</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
-        <v>2018</v>
+        <v>1971</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
@@ -1204,18 +1204,18 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ vào cơ chế lưu KV, cho phép lưu trữ trạng thái của các từ trước đó, giúp mô hình không bị quên thông tin khi chuỗi dữ liệu dài.</t>
+          <t>Transformer giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM nhờ cơ chế lưu KV, cho phép lưu trạng thái của các từ trước đó, giúp mô hình không quên thông tin khi xử lý chuỗi dài.</t>
         </is>
       </c>
       <c r="J12" s="8" t="n">
-        <v>202</v>
+        <v>189</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="L12" s="12" t="inlineStr">
         <is>
-          <t>82.4%</t>
+          <t>83.6%</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
@@ -1226,11 +1226,11 @@
       <c r="N12" s="9" t="inlineStr">
         <is>
           <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
-• Option B: Tại sao RNN và LSTM gặp khó khăn với long-term dependency?</t>
+• Option B: Tại sao việc xử lý song song lại quan trọng trong Transformer?</t>
         </is>
       </c>
       <c r="O12" s="11" t="n">
-        <v>4126</v>
+        <v>2176</v>
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
@@ -1282,33 +1282,33 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Context rot là hiện tượng khi mô hình quên thông tin cũ khi tiếp nhận quá nhiều ngữ cảnh. Việc sử dụng 1 triệu token không đảm bảo độ chính xác cao hơn, vì mô hình có thể mất mát thông tin quan trọng từ đầu vào trước đó.</t>
+          <t>Hiện tượng Context rot xảy ra khi mô hình không thể xử lý thông tin hiệu quả do quá nhiều dữ liệu, dẫn đến việc chú ý sai chỗ. Đưa 1 triệu token có thể làm giảm độ chính xác vì mô hình có thể bị overload và không tập trung vào thông tin quan trọng.</t>
         </is>
       </c>
       <c r="J13" s="8" t="n">
-        <v>220</v>
+        <v>248</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>82.7%</t>
+          <t>80.5%</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-052]</t>
+          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-053]</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao context lại quan trọng trong mô hình ngôn ngữ lớn?
-• Option B: Có cách nào để cải thiện độ chính xác khi sử dụng nhiều token không?</t>
+          <t>• Option A: Tại sao việc quản lý cửa sổ ngữ cảnh lại quan trọng trong AI?
+• Option B: Cách nào để cải thiện độ chính xác khi xử lý nhiều token?</t>
         </is>
       </c>
       <c r="O13" s="11" t="n">
-        <v>2025</v>
+        <v>2274</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
@@ -1360,18 +1360,18 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các mô hình như Prompt Chaining, Routing và Parallelization, giúp chia nhỏ nhiệm vụ, phân loại đầu vào và xử lý song song để tối ưu hóa kết quả.</t>
+          <t>Để duy trì độ chính xác khi mở rộng cửa sổ quan sát, có thể áp dụng các giải pháp như Prompt Chaining, Routing và Parallelization, giúp quản lý và tối ưu hóa quy trình xử lý thông tin.</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>212</v>
+        <v>184</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>77.2%</t>
+          <t>80.2%</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
@@ -1381,12 +1381,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Làm thế nào để xác định khi nào nên sử dụng Routing?
-• Option B: Có những thách thức nào khi áp dụng Parallelization?</t>
+          <t>• Option A: Làm thế nào để áp dụng Prompt Chaining trong thực tế?
+• Option B: Tại sao Routing lại quan trọng trong việc xử lý thông tin?</t>
         </is>
       </c>
       <c r="O14" s="11" t="n">
-        <v>2832</v>
+        <v>1924</v>
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
@@ -1438,18 +1438,18 @@
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Năm 2017, Transformer ra đời với cơ chế Tự chú ý, cho phép mỗi từ trong câu chú ý đến các từ quan trọng khác, giúp mô hình hiểu ngữ cảnh tốt hơn và khắc phục hạn chế của RNN và LSTM trong việc xử lý tuần tự.</t>
+          <t>Transformer, ra mắt năm 2017, là mô hình xử lý ngôn ngữ cho phép mỗi từ chú ý đến các từ quan trọng khác trong câu nhờ cơ chế Attention, giúp hiểu ngữ cảnh tốt hơn và khắc phục nhược điểm của RNN và LSTM.</t>
         </is>
       </c>
       <c r="J15" s="8" t="n">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>-53.3%</t>
+          <t>-51.1%</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
@@ -1459,12 +1459,12 @@
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention hoạt động như thế nào?
-• Option B: So sánh Transformer với RNN và LSTM?</t>
+          <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
+• Option B: So sánh BERT và GPT trong việc xử lý ngôn ngữ.</t>
         </is>
       </c>
       <c r="O15" s="11" t="n">
-        <v>3249</v>
+        <v>2337</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
@@ -1516,33 +1516,33 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention cho phép mỗi từ trong câu 'quay đầu' nhìn lại các từ quan trọng khác, từ đó chấm điểm mức độ liên quan và khóa nghĩa theo ngữ cảnh, giúp mô hình hiểu ngữ nghĩa tốt hơn.</t>
+          <t>Cơ chế Attention trong Transformer cho phép mỗi từ 'nhìn sang' các từ quan trọng khác trong câu, chấm điểm mức độ liên quan và khóa nghĩa theo ngữ cảnh, giúp cải thiện độ chính xác ngữ nghĩa.</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L16" s="12" t="inlineStr">
         <is>
-          <t>-52.9%</t>
+          <t>-57.9%</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 15</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 15 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-040]</t>
         </is>
       </c>
       <c r="N16" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention có ảnh hưởng gì đến việc sinh văn bản không?
-• Option B: Tại sao Attention lại quan trọng hơn các mô hình trước đây?</t>
+          <t>• Option A: Cơ chế Attention có ảnh hưởng như thế nào đến việc xử lý ngôn ngữ tự nhiên?
+• Option B: Tại sao mô hình Transformer lại vượt trội hơn RNN và LSTM?</t>
         </is>
       </c>
       <c r="O16" s="11" t="n">
-        <v>1852</v>
+        <v>2563</v>
       </c>
       <c r="P16" s="12" t="inlineStr">
         <is>
@@ -1594,23 +1594,23 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Self-Attention trong Transformer cho phép xử lý song song toàn bộ ngữ cảnh của các từ, giúp mô hình không quên thông tin từ các từ trước đó, ngay cả khi chuỗi dữ liệu dài.</t>
+          <t>Self-Attention cho phép mỗi token nhìn các token khác trong ngữ cảnh một cách song song, giúp xử lý nhanh chóng và hiệu quả hơn so với các mô hình trước đây như RNN.</t>
         </is>
       </c>
       <c r="J17" s="8" t="n">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L17" s="12" t="inlineStr">
         <is>
-          <t>-52.7%</t>
+          <t>-47.3%</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-06-clean.md] · Đoạn [T06-158]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-06-clean.md] · Đoạn [T06-126]</t>
         </is>
       </c>
       <c r="N17" s="9" t="inlineStr">
@@ -1620,7 +1620,7 @@
         </is>
       </c>
       <c r="O17" s="11" t="n">
-        <v>1933</v>
+        <v>2114</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
@@ -1672,18 +1672,18 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>Năm 2017, Transformer ra đời với cơ chế Attention, cho phép mô hình hiểu ngôn ngữ linh hoạt hơn, không còn bị giới hạn bởi chuỗi tuần tự như RNN hay LSTM. Đây là nền tảng cho các mô hình hiện đại như GPT và BERT.</t>
+          <t>Năm 2017, Transformer ra đời với cơ chế Attention, cho phép mô hình hiểu ngôn ngữ linh hoạt hơn, không còn bị giới hạn bởi chuỗi tuần tự. Đây là nền tảng cho các mô hình như GPT và BERT.</t>
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>212</v>
+        <v>186</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="L18" s="12" t="inlineStr">
         <is>
-          <t>-79.7%</t>
+          <t>-57.6%</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
@@ -1693,12 +1693,12 @@
       </c>
       <c r="N18" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Transformer đã thay đổi cách xử lý ngôn ngữ như thế nào?
-• Option B: BERT và GPT khác nhau ở điểm nào?</t>
+          <t>• Option A: BERT hoạt động như thế nào trong việc hiểu ngôn ngữ?
+• Option B: GPT khác gì so với BERT trong cách sinh văn bản?</t>
         </is>
       </c>
       <c r="O18" s="11" t="n">
-        <v>2128</v>
+        <v>2125</v>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
@@ -1750,33 +1750,33 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Attention trong Transformer xác định các từ quan trọng và tạo ma trận trọng số bằng cách nhận diện mối liên hệ giữa các từ trong câu, từ đó xác định độ liên quan giữa chúng.</t>
+          <t>Cơ chế Attention trong Transformer nhận diện các từ quan trọng và tạo ra ma trận trọng số dựa trên độ liên quan giữa các từ trong câu, giúp mô hình hiểu ngữ cảnh tốt hơn.</t>
         </is>
       </c>
       <c r="J19" s="8" t="n">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="K19" s="11" t="n">
         <v>36</v>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>-94.4%</t>
+          <t>-91.0%</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-054]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-054]</t>
         </is>
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Attention có thể áp dụng cho những loại dữ liệu nào khác không?
-• Option B: Làm thế nào để cải thiện độ chính xác của ma trận trọng số?</t>
+          <t>• Option A: Attention giúp mô hình hiểu ngữ cảnh như thế nào?
+• Option B: Tại sao ma trận trọng số lại quan trọng trong Transformer?</t>
         </is>
       </c>
       <c r="O19" s="11" t="n">
-        <v>1923</v>
+        <v>1941</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
@@ -1828,18 +1828,18 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>BERT là mô hình hiểu ngôn ngữ hai chiều, phân tích ý nghĩa bằng cách xem xét ngữ cảnh từ cả hai phía, trong khi GPT là mô hình sinh văn bản, hoạt động theo chiều từ trái sang phải để dự đoán token tiếp theo.</t>
+          <t>BERT là mô hình hiểu ngôn ngữ hai chiều, phân tích ngữ cảnh từ cả hai phía, trong khi GPT là mô hình sinh văn bản, hoạt động theo chiều từ trái sang phải để dự đoán token tiếp theo.</t>
         </is>
       </c>
       <c r="J20" s="8" t="n">
-        <v>207</v>
+        <v>181</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="L20" s="12" t="inlineStr">
         <is>
-          <t>67.1%</t>
+          <t>71.2%</t>
         </is>
       </c>
       <c r="M20" s="9" t="inlineStr">
@@ -1850,11 +1850,11 @@
       <c r="N20" s="9" t="inlineStr">
         <is>
           <t>• Option A: BERT có thể xử lý ngữ cảnh như thế nào?
-• Option B: GPT có những ứng dụng gì trong thực tế?</t>
+• Option B: GPT hoạt động ra sao trong việc sinh văn bản?</t>
         </is>
       </c>
       <c r="O20" s="11" t="n">
-        <v>2297</v>
+        <v>2251</v>
       </c>
       <c r="P20" s="12" t="inlineStr">
         <is>
@@ -1906,18 +1906,18 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý văn bản trong thẻ, từ đó ngăn chặn hiện tượng Context Bleed và tấn công Prompt Injection.</t>
+          <t>Kỹ thuật Delimiters bao bọc dữ liệu người dùng trong các thẻ định danh rõ ràng, giúp mô hình chỉ xử lý nội dung trong thẻ, từ đó ngăn chặn các câu lệnh độc hại và hiện tượng Context Bleed.</t>
         </is>
       </c>
       <c r="J21" s="8" t="n">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L21" s="12" t="inlineStr">
         <is>
-          <t>78.7%</t>
+          <t>79.1%</t>
         </is>
       </c>
       <c r="M21" s="9" t="inlineStr">
@@ -1927,12 +1927,12 @@
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Có những kỹ thuật nào khác để bảo vệ mô hình khỏi Prompt Injection?
-• Option B: Tại sao Context Bleed lại là vấn đề nghiêm trọng trong AI?</t>
+          <t>• Option A: Delimiters có thể được áp dụng trong trường hợp nào?
+• Option B: Tại sao cần phân định rõ giữa lệnh hệ thống và dữ liệu thô?</t>
         </is>
       </c>
       <c r="O21" s="11" t="n">
-        <v>1978</v>
+        <v>2481</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
@@ -1984,33 +1984,33 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Cơ chế Attention trong Transformer cho phép xử lý song song và lưu trữ trạng thái của các từ trước đó, giúp giải quyết vấn đề long-term dependency tốt hơn RNN và LSTM, vốn chỉ xử lý tuần tự từng từ.</t>
+          <t>Cơ chế Attention giúp mô hình lưu trữ trạng thái của các từ trước đó, cho phép xử lý song song và giảm thiểu hiện tượng quên thông tin trong chuỗi dài, điều mà RNN và LSTM gặp khó khăn.</t>
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>198</v>
+        <v>185</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>84.2%</t>
+          <t>85.2%</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Transcript [transcript-04-clean.md] · Đoạn [T04-094]</t>
+          <t>Slide [d1-slide-hackathon.pdf] · Trang 8 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-094]</t>
         </is>
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Cơ chế Attention hoạt động như thế nào trong Transformer?
-• Option B: So sánh hiệu suất giữa RNN, LSTM và Transformer?</t>
+          <t>• Option A: Cơ chế lưu KV trong Transformer hoạt động như thế nào?
+• Option B: So sánh giữa Attention và RNN trong việc xử lý chuỗi dài?</t>
         </is>
       </c>
       <c r="O22" s="11" t="n">
-        <v>2074</v>
+        <v>2366</v>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="O23" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P23" s="12" t="inlineStr">
         <is>
@@ -2164,7 +2164,7 @@
         </is>
       </c>
       <c r="O24" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
@@ -2216,33 +2216,33 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Khái niệm này đề cập đến việc sử dụng các thẻ định danh để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu, nhằm phân định rõ ràng giữa lệnh hệ thống và dữ liệu thô.</t>
+          <t>Khái niệm này đề cập đến việc sử dụng delimiters để bao bọc dữ liệu từ người dùng, phản hồi API hoặc truy vấn cơ sở dữ liệu trong các thẻ định danh rõ ràng, nhằm ngăn ngừa hiện tượng Context Bleed và tấn công Prompt Injection.</t>
         </is>
       </c>
       <c r="J25" s="8" t="n">
-        <v>189</v>
+        <v>226</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>79.1%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>Slide [d4-slide-hackathon.pdf] · Trang 55</t>
+          <t>Slide [d4-slide-hackathon.pdf] · Trang 55 &amp; Transcript [transcript-04-clean.md] · Đoạn [T04-068]</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong AI?
-• Option B: Có những kỹ thuật nào khác để bảo vệ dữ liệu trong AI?</t>
+          <t>• Option A: Tại sao việc sử dụng delimiters lại quan trọng trong Prompt Engineering?
+• Option B: Context Bleed là gì và tại sao nó cần được ngăn chặn?</t>
         </is>
       </c>
       <c r="O25" s="11" t="n">
-        <v>2167</v>
+        <v>2338</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
@@ -2435,12 +2435,12 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>185.3 ký tự (~40.0 từ - Tóm tắt vi mô PAIR)</t>
+          <t>183.3 ký tự (~39.0 từ - Tóm tắt vi mô PAIR)</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Giảm 82.4% ký tự</t>
+          <t>Giảm 82.6% ký tự</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>2094.7 ms (Đo thực tế qua API GPT-4o-mini)</t>
+          <t>2039.3 ms (Đo thực tế qua API GPT-4o-mini)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">

</xml_diff>